<commit_message>
fix: clear privileged data from Tabella_2026 and Tabelle millesimali in template
</commit_message>
<xml_diff>
--- a/src/siemens_converter/template.xlsx
+++ b/src/siemens_converter/template.xlsx
@@ -6767,7 +6767,6 @@
         <v/>
       </c>
     </row>
-    <row r="249"/>
     <row r="250">
       <c r="A250" s="18" t="n"/>
       <c r="C250" s="189">
@@ -7539,7 +7538,6 @@
       <c r="O282" s="249" t="n"/>
       <c r="P282" s="250" t="n"/>
     </row>
-    <row r="283"/>
     <row r="284">
       <c r="M284" s="235" t="n"/>
     </row>
@@ -7593,7 +7591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A2:H41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="13.2"/>
   <cols>
     <col width="4.109375" customWidth="1" style="137" min="1" max="1"/>
@@ -7609,7 +7607,6 @@
     <col width="9.109375" customWidth="1" style="137" min="11" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="15.6" customHeight="1">
       <c r="A2" s="145" t="n"/>
       <c r="B2" s="150" t="inlineStr">
@@ -7635,9 +7632,7 @@
       </c>
       <c r="C3" s="147" t="n"/>
       <c r="D3" s="147" t="n"/>
-      <c r="E3" s="355" t="n">
-        <v>263.44</v>
-      </c>
+      <c r="E3" s="355" t="n"/>
       <c r="F3" s="242" t="n"/>
     </row>
     <row r="4" ht="15.6" customHeight="1">
@@ -7649,9 +7644,7 @@
       </c>
       <c r="C4" s="147" t="n"/>
       <c r="D4" s="147" t="n"/>
-      <c r="E4" s="356" t="n">
-        <v>2141</v>
-      </c>
+      <c r="E4" s="356" t="n"/>
       <c r="F4" s="242" t="n"/>
       <c r="G4" s="357">
         <f>SUM(E3:E4)</f>
@@ -7667,14 +7660,8 @@
       </c>
       <c r="C5" s="359" t="n"/>
       <c r="D5" s="359" t="n"/>
-      <c r="E5" s="360" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="242" t="inlineStr">
-        <is>
-          <t>prova</t>
-        </is>
-      </c>
+      <c r="E5" s="360" t="n"/>
+      <c r="F5" s="242" t="n"/>
     </row>
     <row r="6" ht="15.6" customHeight="1">
       <c r="A6" s="145" t="n"/>
@@ -7685,9 +7672,7 @@
       </c>
       <c r="C6" s="359" t="n"/>
       <c r="D6" s="359" t="n"/>
-      <c r="E6" s="356" t="n">
-        <v>280</v>
-      </c>
+      <c r="E6" s="356" t="n"/>
       <c r="F6" s="241" t="n"/>
     </row>
     <row r="7" ht="15.6" customHeight="1">
@@ -7699,9 +7684,7 @@
       </c>
       <c r="C7" s="359" t="n"/>
       <c r="D7" s="359" t="n"/>
-      <c r="E7" s="356" t="n">
-        <v>68.2</v>
-      </c>
+      <c r="E7" s="356" t="n"/>
       <c r="F7" s="241" t="n"/>
     </row>
     <row r="8" ht="15.6" customHeight="1">
@@ -7713,9 +7696,7 @@
       </c>
       <c r="C8" s="359" t="n"/>
       <c r="D8" s="359" t="n"/>
-      <c r="E8" s="356" t="n">
-        <v>0</v>
-      </c>
+      <c r="E8" s="356" t="n"/>
       <c r="F8" s="241" t="n"/>
     </row>
     <row r="9" ht="15.6" customHeight="1">
@@ -7806,15 +7787,11 @@
       </c>
     </row>
     <row r="18">
-      <c r="E18" s="144" t="n">
-        <v>45292</v>
-      </c>
-      <c r="F18" s="143" t="n">
-        <v>46022</v>
-      </c>
+      <c r="E18" s="144" t="n"/>
+      <c r="F18" s="143" t="n"/>
       <c r="G18" s="269" t="inlineStr">
         <is>
-          <t>31/??/2026</t>
+          <t>??/??/????</t>
         </is>
       </c>
       <c r="H18" s="142" t="inlineStr">
@@ -7844,12 +7821,8 @@
           <t>Kwh</t>
         </is>
       </c>
-      <c r="F20" s="140" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="223" t="n">
-        <v>1086</v>
-      </c>
+      <c r="F20" s="140" t="n"/>
+      <c r="G20" s="223" t="n"/>
       <c r="H20" s="139">
         <f>G20-F20</f>
         <v/>
@@ -7868,12 +7841,8 @@
           <t>mc</t>
         </is>
       </c>
-      <c r="F21" s="140" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="223" t="n">
-        <v>1718</v>
-      </c>
+      <c r="F21" s="140" t="n"/>
+      <c r="G21" s="223" t="n"/>
       <c r="H21" s="139">
         <f>G21-F21</f>
         <v/>
@@ -7892,12 +7861,8 @@
           <t>mc</t>
         </is>
       </c>
-      <c r="F22" s="140" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="223" t="n">
-        <v>680</v>
-      </c>
+      <c r="F22" s="140" t="n"/>
+      <c r="G22" s="223" t="n"/>
       <c r="H22" s="139">
         <f>G22-F22</f>
         <v/>
@@ -8098,240 +8063,140 @@
       </c>
     </row>
     <row r="4" ht="13.8" customHeight="1">
-      <c r="A4" s="166" t="inlineStr">
-        <is>
-          <t>App, 01 Proprietario 01 /</t>
-        </is>
-      </c>
-      <c r="B4" s="167" t="n">
-        <v>20</v>
-      </c>
-      <c r="C4" s="168" t="n">
-        <v>1344.03</v>
-      </c>
+      <c r="A4" s="166" t="n"/>
+      <c r="B4" s="167" t="n"/>
+      <c r="C4" s="168" t="n"/>
       <c r="D4" s="169">
         <f>C4/$C$3*1000</f>
         <v/>
       </c>
-      <c r="E4" s="170" t="n">
-        <v>1101.36</v>
-      </c>
+      <c r="E4" s="170" t="n"/>
       <c r="F4" s="169">
         <f>+E4/$E$3*1000</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="13.8" customHeight="1">
-      <c r="A5" s="171" t="inlineStr">
-        <is>
-          <t>App, 02 Proprietario 02</t>
-        </is>
-      </c>
-      <c r="B5" s="167" t="n">
-        <v>21</v>
-      </c>
-      <c r="C5" s="170" t="n">
-        <v>2595.68</v>
-      </c>
+      <c r="A5" s="171" t="n"/>
+      <c r="B5" s="167" t="n"/>
+      <c r="C5" s="170" t="n"/>
       <c r="D5" s="169">
         <f>C5/$C$3*1000</f>
         <v/>
       </c>
-      <c r="E5" s="170" t="n">
-        <v>1297.82</v>
-      </c>
+      <c r="E5" s="170" t="n"/>
       <c r="F5" s="169">
         <f>+E5/$E$3*1000</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="13.8" customHeight="1">
-      <c r="A6" s="166" t="inlineStr">
-        <is>
-          <t xml:space="preserve">App, 03 Proprietario 03 / </t>
-        </is>
-      </c>
-      <c r="B6" s="167" t="n">
-        <v>22</v>
-      </c>
-      <c r="C6" s="170" t="n">
-        <v>523.16</v>
-      </c>
+      <c r="A6" s="166" t="n"/>
+      <c r="B6" s="167" t="n"/>
+      <c r="C6" s="170" t="n"/>
       <c r="D6" s="169">
         <f>C6/$C$3*1000</f>
         <v/>
       </c>
-      <c r="E6" s="170" t="n">
-        <v>1090.45</v>
-      </c>
+      <c r="E6" s="170" t="n"/>
       <c r="F6" s="169">
         <f>+E6/$E$3*1000</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="13.8" customHeight="1">
-      <c r="A7" s="171" t="inlineStr">
-        <is>
-          <t>App, 04 Proprietario 02</t>
-        </is>
-      </c>
-      <c r="B7" s="167" t="n">
-        <v>23</v>
-      </c>
-      <c r="C7" s="170" t="n">
-        <v>918.27</v>
-      </c>
+      <c r="A7" s="171" t="n"/>
+      <c r="B7" s="167" t="n"/>
+      <c r="C7" s="170" t="n"/>
       <c r="D7" s="169">
         <f>C7/$C$3*1000</f>
         <v/>
       </c>
-      <c r="E7" s="170" t="n">
-        <v>1204.33</v>
-      </c>
+      <c r="E7" s="170" t="n"/>
       <c r="F7" s="169">
         <f>+E7/$E$3*1000</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="13.8" customHeight="1">
-      <c r="A8" s="171" t="inlineStr">
-        <is>
-          <t>App, 05 Proprietario 02</t>
-        </is>
-      </c>
-      <c r="B8" s="167" t="n">
-        <v>24</v>
-      </c>
-      <c r="C8" s="170" t="n">
-        <v>1353.01</v>
-      </c>
+      <c r="A8" s="171" t="n"/>
+      <c r="B8" s="167" t="n"/>
+      <c r="C8" s="170" t="n"/>
       <c r="D8" s="169">
         <f>C8/$C$3*1000</f>
         <v/>
       </c>
-      <c r="E8" s="170" t="n">
-        <v>1085.06</v>
-      </c>
+      <c r="E8" s="170" t="n"/>
       <c r="F8" s="169">
         <f>+E8/$E$3*1000</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="13.8" customHeight="1">
-      <c r="A9" s="166" t="inlineStr">
-        <is>
-          <t>App, 06 Proprietario 06</t>
-        </is>
-      </c>
-      <c r="B9" s="167" t="n">
-        <v>25</v>
-      </c>
-      <c r="C9" s="170" t="n">
-        <v>332.01</v>
-      </c>
+      <c r="A9" s="166" t="n"/>
+      <c r="B9" s="167" t="n"/>
+      <c r="C9" s="170" t="n"/>
       <c r="D9" s="169">
         <f>C9/$C$3*1000</f>
         <v/>
       </c>
-      <c r="E9" s="170" t="n">
-        <v>1040.11</v>
-      </c>
+      <c r="E9" s="170" t="n"/>
       <c r="F9" s="169">
         <f>+E9/$E$3*1000</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="13.8" customHeight="1">
-      <c r="A10" s="171" t="inlineStr">
-        <is>
-          <t>App, 07 Proprietario 07</t>
-        </is>
-      </c>
-      <c r="B10" s="167" t="n">
-        <v>26</v>
-      </c>
-      <c r="C10" s="170" t="n">
-        <v>624.04</v>
-      </c>
+      <c r="A10" s="171" t="n"/>
+      <c r="B10" s="167" t="n"/>
+      <c r="C10" s="170" t="n"/>
       <c r="D10" s="169">
         <f>C10/$C$3*1000</f>
         <v/>
       </c>
-      <c r="E10" s="170" t="n">
-        <v>1079.15</v>
-      </c>
+      <c r="E10" s="170" t="n"/>
       <c r="F10" s="169">
         <f>+E10/$E$3*1000</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="13.8" customHeight="1">
-      <c r="A11" s="166" t="inlineStr">
-        <is>
-          <t>App, 08 Proprietario 01</t>
-        </is>
-      </c>
-      <c r="B11" s="167" t="n">
-        <v>27</v>
-      </c>
-      <c r="C11" s="170" t="n">
-        <v>722</v>
-      </c>
+      <c r="A11" s="166" t="n"/>
+      <c r="B11" s="167" t="n"/>
+      <c r="C11" s="170" t="n"/>
       <c r="D11" s="169">
         <f>C11/$C$3*1000</f>
         <v/>
       </c>
-      <c r="E11" s="170" t="n">
-        <v>1087.44</v>
-      </c>
+      <c r="E11" s="170" t="n"/>
       <c r="F11" s="169">
         <f>+E11/$E$3*1000</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="13.8" customHeight="1">
-      <c r="A12" s="166" t="inlineStr">
-        <is>
-          <t>App, 09 Proprietario 09</t>
-        </is>
-      </c>
-      <c r="B12" s="167" t="n">
-        <v>28</v>
-      </c>
-      <c r="C12" s="170" t="n">
-        <v>1141.65</v>
-      </c>
+      <c r="A12" s="166" t="n"/>
+      <c r="B12" s="167" t="n"/>
+      <c r="C12" s="170" t="n"/>
       <c r="D12" s="169">
         <f>C12/$C$3*1000</f>
         <v/>
       </c>
-      <c r="E12" s="170" t="n">
-        <v>1090.12</v>
-      </c>
+      <c r="E12" s="170" t="n"/>
       <c r="F12" s="169">
         <f>+E12/$E$3*1000</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="13.8" customHeight="1">
-      <c r="A13" s="171" t="inlineStr">
-        <is>
-          <t>App, 10 Proprietario 07</t>
-        </is>
-      </c>
-      <c r="B13" s="167" t="n">
-        <v>29</v>
-      </c>
-      <c r="C13" s="170" t="n">
-        <v>1656.08</v>
-      </c>
+      <c r="A13" s="171" t="n"/>
+      <c r="B13" s="167" t="n"/>
+      <c r="C13" s="170" t="n"/>
       <c r="D13" s="169">
         <f>C13/$C$3*1000</f>
         <v/>
       </c>
-      <c r="E13" s="170" t="n">
-        <v>1209.74</v>
-      </c>
+      <c r="E13" s="170" t="n"/>
       <c r="F13" s="169">
         <f>+E13/$E$3*1000</f>
         <v/>

</xml_diff>

<commit_message>
feat(writer): populate apartment names from FC_report, add Inquilini sheet
</commit_message>
<xml_diff>
--- a/src/siemens_converter/template.xlsx
+++ b/src/siemens_converter/template.xlsx
@@ -2526,7 +2526,7 @@
     <row r="3">
       <c r="A3" s="232" t="inlineStr">
         <is>
-          <t>App. 01 Proprietario 01 / INQUILINO 01  da 01/09/24</t>
+          <t>App. 01</t>
         </is>
       </c>
       <c r="B3" s="9" t="n"/>
@@ -2542,7 +2542,7 @@
     <row r="4">
       <c r="A4" s="232" t="inlineStr">
         <is>
-          <t>App. 02 Proprietario 02 / INQUILINO 02A dal 15/04/2025</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B4" s="9" t="n"/>
@@ -2558,7 +2558,7 @@
     <row r="5">
       <c r="A5" s="232" t="inlineStr">
         <is>
-          <t>App. 03 Proprietario 03 /  INQUILINO 03  da 01/09/24</t>
+          <t>App. 03</t>
         </is>
       </c>
       <c r="B5" s="9" t="n"/>
@@ -2574,7 +2574,7 @@
     <row r="6">
       <c r="A6" s="232" t="inlineStr">
         <is>
-          <t>App.04 Proprietario 02 /  INQUILINO 04 da 01/03/2025</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B6" s="9" t="n"/>
@@ -2590,7 +2590,7 @@
     <row r="7">
       <c r="A7" s="232" t="inlineStr">
         <is>
-          <t>App. 05 Proprietario 02 /  INQUILINO 05 da 01/05/2025</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B7" s="9" t="n"/>
@@ -2606,7 +2606,7 @@
     <row r="8">
       <c r="A8" s="232" t="inlineStr">
         <is>
-          <t>App. 06 Proprietario 06 / INQUILINO 06 da 01/09/24</t>
+          <t>App. 06</t>
         </is>
       </c>
       <c r="B8" s="9" t="n"/>
@@ -2622,7 +2622,7 @@
     <row r="9">
       <c r="A9" s="232" t="inlineStr">
         <is>
-          <t>App. 07 Proprietario 07 / INQUILINO 07 da 01/03/25</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B9" s="9" t="n"/>
@@ -2638,7 +2638,7 @@
     <row r="10">
       <c r="A10" s="232" t="inlineStr">
         <is>
-          <t>App. 08 Proprietario 01 / INQUILINO 08  da 01/01/26</t>
+          <t>App. 08</t>
         </is>
       </c>
       <c r="B10" s="9" t="n"/>
@@ -2654,7 +2654,7 @@
     <row r="11">
       <c r="A11" s="232" t="inlineStr">
         <is>
-          <t>App. 09 Proprietario 09 /  INQUILINO 09  da 01/11/24</t>
+          <t>App. 09</t>
         </is>
       </c>
       <c r="B11" s="9" t="n"/>
@@ -2670,7 +2670,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>App. 10 Proprietario 07</t>
+          <t>App. 10</t>
         </is>
       </c>
       <c r="B12" s="9" t="n"/>
@@ -3568,11 +3568,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 01</t>
-        </is>
-      </c>
+      <c r="A78" s="200" t="inlineStr"/>
       <c r="B78" s="199" t="n">
         <v>4048</v>
       </c>
@@ -3603,7 +3599,7 @@
     <row r="80">
       <c r="A80" s="200" t="inlineStr">
         <is>
-          <t>App. 02 - Inquilino 02 dal 15/04/2025</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B80" s="199" t="n">
@@ -3632,11 +3628,7 @@
       <c r="G81" s="217" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 03</t>
-        </is>
-      </c>
+      <c r="A82" s="200" t="inlineStr"/>
       <c r="B82" s="199" t="n">
         <v>621</v>
       </c>
@@ -3665,7 +3657,7 @@
     <row r="84">
       <c r="A84" s="200" t="inlineStr">
         <is>
-          <t>App. 04 - Inquilino 04 dal 01/03/2025</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B84" s="199" t="n">
@@ -3696,7 +3688,7 @@
     <row r="86">
       <c r="A86" s="200" t="inlineStr">
         <is>
-          <t>App. 05  INQUILINO 05 dal 01/05/2025</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B86" s="199" t="n">
@@ -3725,11 +3717,7 @@
       <c r="G87" s="217" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 06</t>
-        </is>
-      </c>
+      <c r="A88" s="200" t="inlineStr"/>
       <c r="B88" s="199" t="n">
         <v>169</v>
       </c>
@@ -3758,7 +3746,7 @@
     <row r="90">
       <c r="A90" s="200" t="inlineStr">
         <is>
-          <t>App. 07  Inquilino 07 dal 01/03/2025</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B90" s="199" t="n">
@@ -3787,11 +3775,7 @@
       <c r="G91" s="217" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 08</t>
-        </is>
-      </c>
+      <c r="A92" s="200" t="inlineStr"/>
       <c r="B92" s="199" t="n">
         <v>1708</v>
       </c>
@@ -3818,11 +3802,7 @@
       <c r="E93" s="71" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 09</t>
-        </is>
-      </c>
+      <c r="A94" s="200" t="inlineStr"/>
       <c r="B94" s="199" t="n">
         <v>2720</v>
       </c>
@@ -3953,7 +3933,7 @@
     <row r="102">
       <c r="A102" s="68" t="inlineStr">
         <is>
-          <t>App. 01 Proprietario 01 / INQUILINO 01  da 01/09</t>
+          <t>App. 01</t>
         </is>
       </c>
       <c r="B102" s="83" t="n"/>
@@ -3961,11 +3941,7 @@
       <c r="D102" s="71" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 01</t>
-        </is>
-      </c>
+      <c r="A103" s="200" t="inlineStr"/>
       <c r="B103" s="85">
         <f>+C3</f>
         <v/>
@@ -3983,7 +3959,7 @@
     <row r="104">
       <c r="A104" s="68" t="inlineStr">
         <is>
-          <t xml:space="preserve">App. 02 Proprietario 02 </t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B104" s="83" t="n"/>
@@ -3994,7 +3970,7 @@
     <row r="105">
       <c r="A105" s="200" t="inlineStr">
         <is>
-          <t>App. 02 - Inquilino 02 dal 15/04/2025</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B105" s="85">
@@ -4014,7 +3990,7 @@
     <row r="106">
       <c r="A106" s="68" t="inlineStr">
         <is>
-          <t>App. 03 Proprietario 03 /  INQUILINO 03  da 01/09</t>
+          <t>App. 03</t>
         </is>
       </c>
       <c r="B106" s="83" t="n"/>
@@ -4023,11 +3999,7 @@
       <c r="M106" s="231" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 03</t>
-        </is>
-      </c>
+      <c r="A107" s="200" t="inlineStr"/>
       <c r="B107" s="85">
         <f>+C5</f>
         <v/>
@@ -4045,7 +4017,7 @@
     <row r="108">
       <c r="A108" s="192" t="inlineStr">
         <is>
-          <t>App.04 Proprietario 02</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B108" s="83" t="n"/>
@@ -4056,7 +4028,7 @@
     <row r="109">
       <c r="A109" s="200" t="inlineStr">
         <is>
-          <t>App. 04 - Inquilino 04 dal 01/03/2025</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B109" s="85">
@@ -4077,7 +4049,7 @@
     <row r="110">
       <c r="A110" s="192" t="inlineStr">
         <is>
-          <t>App. 05 Proprietario 02</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B110" s="83" t="n"/>
@@ -4088,7 +4060,7 @@
     <row r="111">
       <c r="A111" s="200" t="inlineStr">
         <is>
-          <t>App. 05  INQUILINO 05 dal 01/05/2025</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B111" s="85">
@@ -4108,7 +4080,7 @@
     <row r="112">
       <c r="A112" s="68" t="inlineStr">
         <is>
-          <t>App. 06 Proprietario 06 / INQUILINO 06 da 01/09</t>
+          <t>App. 06</t>
         </is>
       </c>
       <c r="B112" s="83" t="n"/>
@@ -4117,11 +4089,7 @@
       <c r="M112" s="231" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 06</t>
-        </is>
-      </c>
+      <c r="A113" s="200" t="inlineStr"/>
       <c r="B113" s="85">
         <f>+C8</f>
         <v/>
@@ -4139,7 +4107,7 @@
     <row r="114">
       <c r="A114" s="68" t="inlineStr">
         <is>
-          <t>App. 07 Proprietario 07</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B114" s="83" t="n"/>
@@ -4150,7 +4118,7 @@
     <row r="115">
       <c r="A115" s="200" t="inlineStr">
         <is>
-          <t>App. 07  Inquilino 07 dal 01/03/2025</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B115" s="85">
@@ -4171,7 +4139,7 @@
     <row r="116">
       <c r="A116" s="68" t="inlineStr">
         <is>
-          <t>App. 08 Proprietario 01 / INQUILINO 08  da 01/01/26</t>
+          <t>App. 08</t>
         </is>
       </c>
       <c r="B116" s="83" t="n"/>
@@ -4180,11 +4148,7 @@
       <c r="M116" s="231" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 08</t>
-        </is>
-      </c>
+      <c r="A117" s="200" t="inlineStr"/>
       <c r="B117" s="85">
         <f>+C10</f>
         <v/>
@@ -4202,7 +4166,7 @@
     <row r="118">
       <c r="A118" s="68" t="inlineStr">
         <is>
-          <t>App. 09 Proprietario 09 /  INQUILINO 09  da 01/11</t>
+          <t>App. 09</t>
         </is>
       </c>
       <c r="B118" s="83" t="n"/>
@@ -4211,11 +4175,7 @@
       <c r="M118" s="231" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 09</t>
-        </is>
-      </c>
+      <c r="A119" s="200" t="inlineStr"/>
       <c r="B119" s="85">
         <f>+C11</f>
         <v/>
@@ -4232,7 +4192,7 @@
     <row r="120" ht="13.8" customHeight="1" thickBot="1">
       <c r="A120" s="25" t="inlineStr">
         <is>
-          <t>App. 10 Proprietario 07</t>
+          <t>App. 10</t>
         </is>
       </c>
       <c r="B120" s="87">
@@ -4375,7 +4335,7 @@
     <row r="129">
       <c r="A129" s="68" t="inlineStr">
         <is>
-          <t>App. 01 Proprietario 01 / INQUILINO 01  da 01/09</t>
+          <t>App. 01</t>
         </is>
       </c>
       <c r="B129" s="328" t="n"/>
@@ -4385,11 +4345,7 @@
       <c r="F129" s="71" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 01</t>
-        </is>
-      </c>
+      <c r="A130" s="200" t="inlineStr"/>
       <c r="B130" s="330" t="n">
         <v>28.114</v>
       </c>
@@ -4412,7 +4368,7 @@
     <row r="131">
       <c r="A131" s="68" t="inlineStr">
         <is>
-          <t>App. 02 Proprietario 02 / INQUILINO 02</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B131" s="328" t="n"/>
@@ -4426,7 +4382,7 @@
     <row r="132" ht="14.4" customHeight="1">
       <c r="A132" s="200" t="inlineStr">
         <is>
-          <t>App. 02 - Inquilino 02 dal 15/04/2025</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B132" s="330" t="n">
@@ -4451,7 +4407,7 @@
     <row r="133">
       <c r="A133" s="68" t="inlineStr">
         <is>
-          <t>App. 03 Proprietario 03 /  INQUILINO 03  da 01/09</t>
+          <t>App. 03</t>
         </is>
       </c>
       <c r="B133" s="328" t="n"/>
@@ -4461,11 +4417,7 @@
       <c r="F133" s="71" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 03</t>
-        </is>
-      </c>
+      <c r="A134" s="200" t="inlineStr"/>
       <c r="B134" s="330" t="n">
         <v>38.014</v>
       </c>
@@ -4488,7 +4440,7 @@
     <row r="135">
       <c r="A135" s="192" t="inlineStr">
         <is>
-          <t>App.04 Proprietario 02</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B135" s="328" t="n"/>
@@ -4500,7 +4452,7 @@
     <row r="136" ht="14.4" customHeight="1">
       <c r="A136" s="200" t="inlineStr">
         <is>
-          <t>App. 04 - Inquilino 04</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B136" s="330" t="n">
@@ -4525,7 +4477,7 @@
     <row r="137">
       <c r="A137" s="192" t="inlineStr">
         <is>
-          <t>App. 05 Proprietario 02</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B137" s="328" t="n"/>
@@ -4538,7 +4490,7 @@
     <row r="138" ht="14.4" customHeight="1">
       <c r="A138" s="200" t="inlineStr">
         <is>
-          <t>App. 05  INQUILINO 05 dal 01/05/2025</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B138" s="330" t="n">
@@ -4563,7 +4515,7 @@
     <row r="139">
       <c r="A139" s="68" t="inlineStr">
         <is>
-          <t>App. 06 Proprietario 06 / INQUILINO 06 da 01/09</t>
+          <t>App. 06</t>
         </is>
       </c>
       <c r="B139" s="328" t="n"/>
@@ -4573,11 +4525,7 @@
       <c r="F139" s="71" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 06</t>
-        </is>
-      </c>
+      <c r="A140" s="200" t="inlineStr"/>
       <c r="B140" s="330" t="n">
         <v>17.497</v>
       </c>
@@ -4600,7 +4548,7 @@
     <row r="141">
       <c r="A141" s="68" t="inlineStr">
         <is>
-          <t>App. 07 Proprietario 07</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B141" s="328" t="n"/>
@@ -4613,7 +4561,7 @@
     <row r="142" ht="14.4" customHeight="1">
       <c r="A142" s="200" t="inlineStr">
         <is>
-          <t>App. 07  Inquilino 07</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B142" s="330" t="n">
@@ -4638,7 +4586,7 @@
     <row r="143">
       <c r="A143" s="68" t="inlineStr">
         <is>
-          <t>App. 08 Proprietario 01 / INQUILINO 08  da 01/01/26</t>
+          <t>App. 08</t>
         </is>
       </c>
       <c r="B143" s="328" t="n"/>
@@ -4648,11 +4596,7 @@
       <c r="F143" s="71" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 08</t>
-        </is>
-      </c>
+      <c r="A144" s="200" t="inlineStr"/>
       <c r="B144" s="330" t="n">
         <v>102.587</v>
       </c>
@@ -4675,7 +4619,7 @@
     <row r="145">
       <c r="A145" s="68" t="inlineStr">
         <is>
-          <t>App. 09 Proprietario 09 /  INQUILINO 09  da 01/11</t>
+          <t>App. 09</t>
         </is>
       </c>
       <c r="B145" s="328" t="n"/>
@@ -4685,11 +4629,7 @@
       <c r="F145" s="71" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 09</t>
-        </is>
-      </c>
+      <c r="A146" s="200" t="inlineStr"/>
       <c r="B146" s="330" t="n">
         <v>69.572</v>
       </c>
@@ -4712,7 +4652,7 @@
     <row r="147" ht="13.8" customHeight="1" thickBot="1">
       <c r="A147" s="25" t="inlineStr">
         <is>
-          <t>App. 10 Proprietario 07</t>
+          <t>App. 10</t>
         </is>
       </c>
       <c r="B147" s="335" t="n">
@@ -4873,7 +4813,7 @@
     <row r="157">
       <c r="A157" s="68" t="inlineStr">
         <is>
-          <t>App. 01 Proprietario 01 / INQUILINO 01  da 01/09</t>
+          <t>App. 01</t>
         </is>
       </c>
       <c r="B157" s="83" t="n"/>
@@ -4881,11 +4821,7 @@
       <c r="D157" s="71" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 01</t>
-        </is>
-      </c>
+      <c r="A158" s="200" t="inlineStr"/>
       <c r="B158" s="85">
         <f>D3</f>
         <v/>
@@ -4902,7 +4838,7 @@
     <row r="159">
       <c r="A159" s="68" t="inlineStr">
         <is>
-          <t>App. 02 Proprietario 02 / INQUILINO 02+A194</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B159" s="83" t="n"/>
@@ -4912,7 +4848,7 @@
     <row r="160">
       <c r="A160" s="200" t="inlineStr">
         <is>
-          <t>App. 02 - Inquilino 02 dal 15/04/2025</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B160" s="85">
@@ -4931,7 +4867,7 @@
     <row r="161">
       <c r="A161" s="68" t="inlineStr">
         <is>
-          <t>App. 03 Proprietario 03 /  INQUILINO 03  da 01/09</t>
+          <t>App. 03</t>
         </is>
       </c>
       <c r="B161" s="83" t="n"/>
@@ -4939,11 +4875,7 @@
       <c r="D161" s="71" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 03</t>
-        </is>
-      </c>
+      <c r="A162" s="200" t="inlineStr"/>
       <c r="B162" s="85">
         <f>D5</f>
         <v/>
@@ -4961,7 +4893,7 @@
     <row r="163">
       <c r="A163" s="192" t="inlineStr">
         <is>
-          <t>App.04 Proprietario 02</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B163" s="83" t="n"/>
@@ -4971,7 +4903,7 @@
     <row r="164">
       <c r="A164" s="200" t="inlineStr">
         <is>
-          <t>App. 04 - Inquilino 04</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B164" s="85">
@@ -4991,7 +4923,7 @@
     <row r="165">
       <c r="A165" s="192" t="inlineStr">
         <is>
-          <t>App. 05 Proprietario 02</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B165" s="83" t="n"/>
@@ -5001,7 +4933,7 @@
     <row r="166">
       <c r="A166" s="200" t="inlineStr">
         <is>
-          <t>App. 05  INQUILINO 05 dal 01/05/2025</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B166" s="85">
@@ -5020,7 +4952,7 @@
     <row r="167">
       <c r="A167" s="68" t="inlineStr">
         <is>
-          <t>App. 06 Proprietario 06 / INQUILINO 06 da 01/09</t>
+          <t>App. 06</t>
         </is>
       </c>
       <c r="B167" s="83" t="n"/>
@@ -5028,11 +4960,7 @@
       <c r="D167" s="71" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 06</t>
-        </is>
-      </c>
+      <c r="A168" s="200" t="inlineStr"/>
       <c r="B168" s="85">
         <f>D8</f>
         <v/>
@@ -5049,7 +4977,7 @@
     <row r="169">
       <c r="A169" s="68" t="inlineStr">
         <is>
-          <t>App. 07 Proprietario 07</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B169" s="83" t="n"/>
@@ -5059,7 +4987,7 @@
     <row r="170">
       <c r="A170" s="200" t="inlineStr">
         <is>
-          <t>App. 07  Inquilino 07</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B170" s="85">
@@ -5079,7 +5007,7 @@
     <row r="171">
       <c r="A171" s="68" t="inlineStr">
         <is>
-          <t>App. 08 Proprietario 01 / INQUILINO 08  da 01/01/26</t>
+          <t>App. 08</t>
         </is>
       </c>
       <c r="B171" s="83" t="n"/>
@@ -5087,11 +5015,7 @@
       <c r="D171" s="71" t="n"/>
     </row>
     <row r="172">
-      <c r="A172" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 08</t>
-        </is>
-      </c>
+      <c r="A172" s="200" t="inlineStr"/>
       <c r="B172" s="85">
         <f>D10</f>
         <v/>
@@ -5108,7 +5032,7 @@
     <row r="173">
       <c r="A173" s="68" t="inlineStr">
         <is>
-          <t>App. 09 Proprietario 09 /  INQUILINO 09  da 01/11</t>
+          <t>App. 09</t>
         </is>
       </c>
       <c r="B173" s="83" t="n"/>
@@ -5116,11 +5040,7 @@
       <c r="D173" s="71" t="n"/>
     </row>
     <row r="174" ht="13.8" customHeight="1" thickBot="1">
-      <c r="A174" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 09</t>
-        </is>
-      </c>
+      <c r="A174" s="200" t="inlineStr"/>
       <c r="B174" s="85">
         <f>D11</f>
         <v/>
@@ -5137,7 +5057,7 @@
     <row r="175" ht="13.8" customHeight="1" thickBot="1">
       <c r="A175" s="25" t="inlineStr">
         <is>
-          <t>App. 10 Proprietario 07</t>
+          <t>App. 10</t>
         </is>
       </c>
       <c r="B175" s="87">
@@ -5256,7 +5176,7 @@
     <row r="181">
       <c r="A181" s="68" t="inlineStr">
         <is>
-          <t>App. 01 Proprietario 01 / INQUILINO 01  da 01/09</t>
+          <t>App. 01</t>
         </is>
       </c>
       <c r="B181" s="328" t="n"/>
@@ -5267,11 +5187,7 @@
       <c r="G181" s="82" t="n"/>
     </row>
     <row r="182">
-      <c r="A182" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 01</t>
-        </is>
-      </c>
+      <c r="A182" s="200" t="inlineStr"/>
       <c r="B182" s="330" t="n">
         <v>42.48</v>
       </c>
@@ -5293,7 +5209,7 @@
     <row r="183">
       <c r="A183" s="68" t="inlineStr">
         <is>
-          <t>App. 02 Proprietario 02 / INQUILINO 02</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B183" s="328" t="n"/>
@@ -5306,7 +5222,7 @@
     <row r="184">
       <c r="A184" s="200" t="inlineStr">
         <is>
-          <t>App. 02 - Inquilino 02 dal 15/04/2025</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B184" s="330" t="n">
@@ -5330,7 +5246,7 @@
     <row r="185">
       <c r="A185" s="68" t="inlineStr">
         <is>
-          <t>App. 03 Proprietario 03 /  INQUILINO 03  da 01/09</t>
+          <t>App. 03</t>
         </is>
       </c>
       <c r="B185" s="328" t="n"/>
@@ -5341,11 +5257,7 @@
       <c r="G185" s="82" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 03</t>
-        </is>
-      </c>
+      <c r="A186" s="200" t="inlineStr"/>
       <c r="B186" s="341" t="n">
         <v>67</v>
       </c>
@@ -5373,7 +5285,7 @@
     <row r="187">
       <c r="A187" s="190" t="inlineStr">
         <is>
-          <t>App.04 Proprietario 02</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B187" s="328" t="n"/>
@@ -5386,7 +5298,7 @@
     <row r="188">
       <c r="A188" s="200" t="inlineStr">
         <is>
-          <t>App. 04 - Inquilino 04</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B188" s="330" t="n">
@@ -5410,7 +5322,7 @@
     <row r="189">
       <c r="A189" s="192" t="inlineStr">
         <is>
-          <t>App. 05 Proprietario 02</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B189" s="328" t="n"/>
@@ -5423,7 +5335,7 @@
     <row r="190">
       <c r="A190" s="200" t="inlineStr">
         <is>
-          <t>App. 05  INQUILINO 05 dal 01/05/2025</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B190" s="330" t="n">
@@ -5447,7 +5359,7 @@
     <row r="191">
       <c r="A191" s="68" t="inlineStr">
         <is>
-          <t>App. 06 Proprietario 06 / INQUILINO 06 da 01/09</t>
+          <t>App. 06</t>
         </is>
       </c>
       <c r="B191" s="328" t="n"/>
@@ -5458,11 +5370,7 @@
       <c r="G191" s="82" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 06</t>
-        </is>
-      </c>
+      <c r="A192" s="200" t="inlineStr"/>
       <c r="B192" s="330" t="n">
         <v>19.67</v>
       </c>
@@ -5484,7 +5392,7 @@
     <row r="193">
       <c r="A193" s="68" t="inlineStr">
         <is>
-          <t>App. 07 Proprietario 07</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B193" s="328" t="n"/>
@@ -5497,7 +5405,7 @@
     <row r="194">
       <c r="A194" s="200" t="inlineStr">
         <is>
-          <t>App. 07  Inquilino 07</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B194" s="330" t="n">
@@ -5521,7 +5429,7 @@
     <row r="195">
       <c r="A195" s="68" t="inlineStr">
         <is>
-          <t>App. 08 Proprietario 01 / INQUILINO 08  da 01/01/26</t>
+          <t>App. 08</t>
         </is>
       </c>
       <c r="B195" s="328" t="n"/>
@@ -5535,11 +5443,7 @@
       <c r="G195" s="82" t="n"/>
     </row>
     <row r="196">
-      <c r="A196" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 08</t>
-        </is>
-      </c>
+      <c r="A196" s="200" t="inlineStr"/>
       <c r="B196" s="330" t="n">
         <v>88.23999999999999</v>
       </c>
@@ -5561,7 +5465,7 @@
     <row r="197">
       <c r="A197" s="68" t="inlineStr">
         <is>
-          <t>App. 09 Proprietario 09 /  INQUILINO 09  da 01/11</t>
+          <t>App. 09</t>
         </is>
       </c>
       <c r="B197" s="328" t="n"/>
@@ -5575,11 +5479,7 @@
       <c r="G197" s="82" t="n"/>
     </row>
     <row r="198">
-      <c r="A198" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 09</t>
-        </is>
-      </c>
+      <c r="A198" s="200" t="inlineStr"/>
       <c r="B198" s="330" t="n">
         <v>51.03</v>
       </c>
@@ -5601,7 +5501,7 @@
     <row r="199" ht="13.8" customHeight="1" thickBot="1">
       <c r="A199" s="25" t="inlineStr">
         <is>
-          <t>App. 10 Proprietario 07</t>
+          <t>App. 10</t>
         </is>
       </c>
       <c r="B199" s="335" t="n">
@@ -5700,17 +5600,13 @@
     <row r="204">
       <c r="A204" s="68" t="inlineStr">
         <is>
-          <t>App. 01 Proprietario 01 / INQUILINO 01  da 01/09</t>
+          <t>App. 01</t>
         </is>
       </c>
       <c r="E204" s="80" t="n"/>
     </row>
     <row r="205">
-      <c r="A205" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 01</t>
-        </is>
-      </c>
+      <c r="A205" s="200" t="inlineStr"/>
       <c r="B205" s="279">
         <f>+C3</f>
         <v/>
@@ -5731,7 +5627,7 @@
     <row r="206">
       <c r="A206" s="68" t="inlineStr">
         <is>
-          <t>App. 02 Proprietario 02</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="E206" s="80" t="n"/>
@@ -5739,7 +5635,7 @@
     <row r="207">
       <c r="A207" s="200" t="inlineStr">
         <is>
-          <t>App. 02 - Inquilino 02</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B207" s="279">
@@ -5762,17 +5658,13 @@
     <row r="208">
       <c r="A208" s="68" t="inlineStr">
         <is>
-          <t>App. 03 Proprietario 03 /  INQUILINO 03  da 01/09</t>
+          <t>App. 03</t>
         </is>
       </c>
       <c r="E208" s="80" t="n"/>
     </row>
     <row r="209">
-      <c r="A209" s="72" t="inlineStr">
-        <is>
-          <t>INQUILINO 03</t>
-        </is>
-      </c>
+      <c r="A209" s="72" t="inlineStr"/>
       <c r="B209" s="279">
         <f>+C5</f>
         <v/>
@@ -5793,7 +5685,7 @@
     <row r="210">
       <c r="A210" s="192" t="inlineStr">
         <is>
-          <t>App.04 Proprietario 02</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="E210" s="80" t="n"/>
@@ -5801,7 +5693,7 @@
     <row r="211">
       <c r="A211" s="200" t="inlineStr">
         <is>
-          <t>App. 04 - Inquilino 04</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B211" s="279">
@@ -5824,7 +5716,7 @@
     <row r="212">
       <c r="A212" s="192" t="inlineStr">
         <is>
-          <t>App. 05 Proprietario 02</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="E212" s="80" t="n"/>
@@ -5832,7 +5724,7 @@
     <row r="213">
       <c r="A213" s="200" t="inlineStr">
         <is>
-          <t>App. 05  INQUILINO 05 dal 01/05/2025</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B213" s="279">
@@ -5855,17 +5747,13 @@
     <row r="214">
       <c r="A214" s="68" t="inlineStr">
         <is>
-          <t>App. 06 Proprietario 06 / INQUILINO 06 da 01/09</t>
+          <t>App. 06</t>
         </is>
       </c>
       <c r="E214" s="80" t="n"/>
     </row>
     <row r="215">
-      <c r="A215" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 06</t>
-        </is>
-      </c>
+      <c r="A215" s="200" t="inlineStr"/>
       <c r="B215" s="279">
         <f>+C8</f>
         <v/>
@@ -5886,7 +5774,7 @@
     <row r="216">
       <c r="A216" s="68" t="inlineStr">
         <is>
-          <t>App. 07 Proprietario 07</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="E216" s="80" t="n"/>
@@ -5894,7 +5782,7 @@
     <row r="217">
       <c r="A217" s="200" t="inlineStr">
         <is>
-          <t>App. 07  Inquilino 07</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B217" s="279">
@@ -5917,17 +5805,13 @@
     <row r="218">
       <c r="A218" s="68" t="inlineStr">
         <is>
-          <t>App. 08 Proprietario 01 / INQUILINO 08  da 01/01/26</t>
+          <t>App. 08</t>
         </is>
       </c>
       <c r="E218" s="80" t="n"/>
     </row>
     <row r="219">
-      <c r="A219" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 08</t>
-        </is>
-      </c>
+      <c r="A219" s="200" t="inlineStr"/>
       <c r="B219" s="279">
         <f>+C10</f>
         <v/>
@@ -5948,17 +5832,13 @@
     <row r="220">
       <c r="A220" s="68" t="inlineStr">
         <is>
-          <t>App. 09 Proprietario 09 /  INQUILINO 09  da 01/11</t>
+          <t>App. 09</t>
         </is>
       </c>
       <c r="E220" s="80" t="n"/>
     </row>
     <row r="221">
-      <c r="A221" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 09</t>
-        </is>
-      </c>
+      <c r="A221" s="200" t="inlineStr"/>
       <c r="B221" s="279">
         <f>+C11</f>
         <v/>
@@ -5979,7 +5859,7 @@
     <row r="222" ht="13.8" customHeight="1" thickBot="1">
       <c r="A222" s="25" t="inlineStr">
         <is>
-          <t>App. 10 Proprietario 07</t>
+          <t>App. 10</t>
         </is>
       </c>
       <c r="B222" s="277">
@@ -6148,7 +6028,7 @@
     <row r="228">
       <c r="A228" s="68" t="inlineStr">
         <is>
-          <t>App. 01 Proprietario 01 / INQUILINO 01  da 01/09/24</t>
+          <t>App. 01</t>
         </is>
       </c>
       <c r="B228" s="123" t="n"/>
@@ -6164,11 +6044,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 01</t>
-        </is>
-      </c>
+      <c r="A229" s="200" t="inlineStr"/>
       <c r="B229" s="126">
         <f>+F130</f>
         <v/>
@@ -6205,7 +6081,7 @@
     <row r="230">
       <c r="A230" s="68" t="inlineStr">
         <is>
-          <t>App. 02 Proprietario 02 / INQUILINO 02</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B230" s="123" t="n"/>
@@ -6223,7 +6099,7 @@
     <row r="231">
       <c r="A231" s="200" t="inlineStr">
         <is>
-          <t>App. 02 - Inquilino 02 dal 15/04/25</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B231" s="126">
@@ -6262,7 +6138,7 @@
     <row r="232">
       <c r="A232" s="68" t="inlineStr">
         <is>
-          <t>App. 03 Proprietario 03 /  INQUILINO 03  da 01/09/24</t>
+          <t>App. 03</t>
         </is>
       </c>
       <c r="B232" s="123" t="n"/>
@@ -6278,11 +6154,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 03</t>
-        </is>
-      </c>
+      <c r="A233" s="200" t="inlineStr"/>
       <c r="B233" s="126">
         <f>+F134</f>
         <v/>
@@ -6319,7 +6191,7 @@
     <row r="234">
       <c r="A234" s="68" t="inlineStr">
         <is>
-          <t>App.04 Proprietario 02</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B234" s="123" t="n"/>
@@ -6337,7 +6209,7 @@
     <row r="235">
       <c r="A235" s="200" t="inlineStr">
         <is>
-          <t>App. 04 - Inquilino 04 dal 01/03/25</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B235" s="126">
@@ -6376,7 +6248,7 @@
     <row r="236">
       <c r="A236" s="192" t="inlineStr">
         <is>
-          <t>App. 05 Proprietario 02</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B236" s="123" t="n"/>
@@ -6394,7 +6266,7 @@
     <row r="237">
       <c r="A237" s="200" t="inlineStr">
         <is>
-          <t>App. 05  Inquilino 05 dal 01/05/25</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B237" s="126">
@@ -6433,7 +6305,7 @@
     <row r="238">
       <c r="A238" s="68" t="inlineStr">
         <is>
-          <t>App. 06 Proprietario 06 / INQUILINO 06 da 01/09/24</t>
+          <t>App. 06</t>
         </is>
       </c>
       <c r="B238" s="123" t="n"/>
@@ -6449,11 +6321,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 06</t>
-        </is>
-      </c>
+      <c r="A239" s="200" t="inlineStr"/>
       <c r="B239" s="126">
         <f>+F140</f>
         <v/>
@@ -6490,7 +6358,7 @@
     <row r="240">
       <c r="A240" s="68" t="inlineStr">
         <is>
-          <t>App. 07 Proprietario 07</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B240" s="123" t="n"/>
@@ -6508,7 +6376,7 @@
     <row r="241">
       <c r="A241" s="200" t="inlineStr">
         <is>
-          <t>App. 07  Inquilino 07 dal 01/03/25</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B241" s="126">
@@ -6547,7 +6415,7 @@
     <row r="242">
       <c r="A242" s="68" t="inlineStr">
         <is>
-          <t>App. 08 Proprietario 01 / INQUILINO 08  da 01/01/26</t>
+          <t>App. 08</t>
         </is>
       </c>
       <c r="B242" s="123" t="n"/>
@@ -6564,11 +6432,7 @@
       <c r="K242" s="56" t="n"/>
     </row>
     <row r="243">
-      <c r="A243" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 08</t>
-        </is>
-      </c>
+      <c r="A243" s="200" t="inlineStr"/>
       <c r="B243" s="126">
         <f>+F144</f>
         <v/>
@@ -6606,7 +6470,7 @@
     <row r="244">
       <c r="A244" s="68" t="inlineStr">
         <is>
-          <t>App. 09 Proprietario 09 /  INQUILINO 09  da 01/11/24</t>
+          <t>App. 09</t>
         </is>
       </c>
       <c r="B244" s="123" t="n"/>
@@ -6623,11 +6487,7 @@
       <c r="K244" s="56" t="n"/>
     </row>
     <row r="245">
-      <c r="A245" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 09</t>
-        </is>
-      </c>
+      <c r="A245" s="200" t="inlineStr"/>
       <c r="B245" s="126">
         <f>+F146</f>
         <v/>
@@ -6665,7 +6525,7 @@
     <row r="246" ht="13.8" customHeight="1" thickBot="1">
       <c r="A246" s="25" t="inlineStr">
         <is>
-          <t>App. 10 Proprietario 07</t>
+          <t>App. 10</t>
         </is>
       </c>
       <c r="B246" s="129">
@@ -6767,6 +6627,7 @@
         <v/>
       </c>
     </row>
+    <row r="249"/>
     <row r="250">
       <c r="A250" s="18" t="n"/>
       <c r="C250" s="189">
@@ -6968,7 +6829,7 @@
     <row r="258">
       <c r="A258" s="68" t="inlineStr">
         <is>
-          <t>App. 01 Proprietario 01 / INQUILINO 01  da 01/09/24</t>
+          <t>App. 01</t>
         </is>
       </c>
       <c r="B258" s="123" t="n"/>
@@ -6985,11 +6846,7 @@
       <c r="P258" s="80" t="n"/>
     </row>
     <row r="259">
-      <c r="A259" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 01</t>
-        </is>
-      </c>
+      <c r="A259" s="200" t="inlineStr"/>
       <c r="B259" s="126" t="n"/>
       <c r="C259" s="127" t="n"/>
       <c r="D259" s="126" t="n"/>
@@ -7007,7 +6864,7 @@
     <row r="260">
       <c r="A260" s="68" t="inlineStr">
         <is>
-          <t>App. 02 Proprietario 02 / INQUILINO 02</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B260" s="123" t="n"/>
@@ -7027,7 +6884,7 @@
     <row r="261" ht="14.4" customHeight="1">
       <c r="A261" s="200" t="inlineStr">
         <is>
-          <t>App. 02 - Inquilino 02 dal 15/04/25</t>
+          <t>App. 02</t>
         </is>
       </c>
       <c r="B261" s="126" t="n"/>
@@ -7063,7 +6920,7 @@
     <row r="262">
       <c r="A262" s="68" t="inlineStr">
         <is>
-          <t>App. 03 Proprietario 03 /  INQUILINO 03  da 01/09/24</t>
+          <t>App. 03</t>
         </is>
       </c>
       <c r="B262" s="123" t="n"/>
@@ -7082,11 +6939,7 @@
       <c r="P262" s="80" t="n"/>
     </row>
     <row r="263">
-      <c r="A263" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 03</t>
-        </is>
-      </c>
+      <c r="A263" s="200" t="inlineStr"/>
       <c r="B263" s="126" t="n"/>
       <c r="C263" s="127" t="n"/>
       <c r="D263" s="126" t="n"/>
@@ -7105,7 +6958,7 @@
     <row r="264">
       <c r="A264" s="68" t="inlineStr">
         <is>
-          <t>App.04 Proprietario 02</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B264" s="123" t="n"/>
@@ -7126,7 +6979,7 @@
     <row r="265" ht="14.4" customHeight="1">
       <c r="A265" s="200" t="inlineStr">
         <is>
-          <t>App. 04 - Inquilino 04 dal 01/03/25</t>
+          <t>App. 04</t>
         </is>
       </c>
       <c r="B265" s="126" t="n"/>
@@ -7162,7 +7015,7 @@
     <row r="266">
       <c r="A266" s="192" t="inlineStr">
         <is>
-          <t>App. 05 Proprietario 02</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B266" s="123" t="n"/>
@@ -7188,7 +7041,7 @@
     <row r="267" ht="14.4" customHeight="1">
       <c r="A267" s="200" t="inlineStr">
         <is>
-          <t>App. 05  Inquilino 05 dal 01/05/25</t>
+          <t>App. 05</t>
         </is>
       </c>
       <c r="B267" s="126" t="n"/>
@@ -7229,7 +7082,7 @@
     <row r="268">
       <c r="A268" s="68" t="inlineStr">
         <is>
-          <t>App. 06 Proprietario 06 / INQUILINO 06 da 01/09/24</t>
+          <t>App. 06</t>
         </is>
       </c>
       <c r="B268" s="123" t="n"/>
@@ -7248,11 +7101,7 @@
       <c r="P268" s="80" t="n"/>
     </row>
     <row r="269">
-      <c r="A269" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 06</t>
-        </is>
-      </c>
+      <c r="A269" s="200" t="inlineStr"/>
       <c r="B269" s="126" t="n"/>
       <c r="C269" s="127" t="n"/>
       <c r="D269" s="126" t="n"/>
@@ -7271,7 +7120,7 @@
     <row r="270">
       <c r="A270" s="68" t="inlineStr">
         <is>
-          <t>App. 07 Proprietario 07</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B270" s="123" t="n"/>
@@ -7292,7 +7141,7 @@
     <row r="271" ht="14.4" customHeight="1">
       <c r="A271" s="200" t="inlineStr">
         <is>
-          <t>App. 07  Inquilino 07 dal 01/03/25</t>
+          <t>App. 07</t>
         </is>
       </c>
       <c r="B271" s="126" t="n"/>
@@ -7328,7 +7177,7 @@
     <row r="272">
       <c r="A272" s="68" t="inlineStr">
         <is>
-          <t>App. 08 Proprietario 01 / INQUILINO 08  da 01/01/26</t>
+          <t>App. 08</t>
         </is>
       </c>
       <c r="B272" s="123" t="n"/>
@@ -7346,11 +7195,7 @@
       <c r="P272" s="80" t="n"/>
     </row>
     <row r="273" ht="14.4" customHeight="1">
-      <c r="A273" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 08</t>
-        </is>
-      </c>
+      <c r="A273" s="200" t="inlineStr"/>
       <c r="B273" s="126" t="n"/>
       <c r="C273" s="127" t="n"/>
       <c r="D273" s="126" t="n"/>
@@ -7379,7 +7224,7 @@
     <row r="274">
       <c r="A274" s="68" t="inlineStr">
         <is>
-          <t>App. 09 Proprietario 09 /  INQUILINO 09  da 01/11/24</t>
+          <t>App. 09</t>
         </is>
       </c>
       <c r="B274" s="123" t="n"/>
@@ -7397,11 +7242,7 @@
       <c r="P274" s="80" t="n"/>
     </row>
     <row r="275">
-      <c r="A275" s="200" t="inlineStr">
-        <is>
-          <t>INQUILINO 09</t>
-        </is>
-      </c>
+      <c r="A275" s="200" t="inlineStr"/>
       <c r="B275" s="126" t="n"/>
       <c r="C275" s="127" t="n"/>
       <c r="D275" s="126" t="n"/>
@@ -7419,7 +7260,7 @@
     <row r="276" ht="13.8" customHeight="1" thickBot="1">
       <c r="A276" s="25" t="inlineStr">
         <is>
-          <t>App. 10 Proprietario 07</t>
+          <t>App. 10</t>
         </is>
       </c>
       <c r="B276" s="129" t="n"/>
@@ -7538,6 +7379,7 @@
       <c r="O282" s="249" t="n"/>
       <c r="P282" s="250" t="n"/>
     </row>
+    <row r="283"/>
     <row r="284">
       <c r="M284" s="235" t="n"/>
     </row>

</xml_diff>

<commit_message>
fix(writer): tenant rows reference Inquilini sheet via formulas, apartment names only on summary rows
</commit_message>
<xml_diff>
--- a/src/siemens_converter/template.xlsx
+++ b/src/siemens_converter/template.xlsx
@@ -3568,7 +3568,10 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="200" t="inlineStr"/>
+      <c r="A78" s="200">
+        <f>Inquilini!B2</f>
+        <v/>
+      </c>
       <c r="B78" s="199" t="n">
         <v>4048</v>
       </c>
@@ -3597,10 +3600,9 @@
       <c r="G79" s="217" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="200" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A80" s="200">
+        <f>Inquilini!B3</f>
+        <v/>
       </c>
       <c r="B80" s="199" t="n">
         <v>4727</v>
@@ -3628,7 +3630,10 @@
       <c r="G81" s="217" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="200" t="inlineStr"/>
+      <c r="A82" s="200">
+        <f>Inquilini!B4</f>
+        <v/>
+      </c>
       <c r="B82" s="199" t="n">
         <v>621</v>
       </c>
@@ -3655,10 +3660,9 @@
       <c r="G83" s="217" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="200" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A84" s="200">
+        <f>Inquilini!B5</f>
+        <v/>
       </c>
       <c r="B84" s="199" t="n">
         <v>922</v>
@@ -3686,10 +3690,9 @@
       <c r="G85" s="217" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="200" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A86" s="200">
+        <f>Inquilini!B6</f>
+        <v/>
       </c>
       <c r="B86" s="199" t="n">
         <v>102</v>
@@ -3717,7 +3720,10 @@
       <c r="G87" s="217" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="200" t="inlineStr"/>
+      <c r="A88" s="200">
+        <f>Inquilini!B7</f>
+        <v/>
+      </c>
       <c r="B88" s="199" t="n">
         <v>169</v>
       </c>
@@ -3744,10 +3750,9 @@
       <c r="G89" s="217" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="200" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A90" s="200">
+        <f>Inquilini!B8</f>
+        <v/>
       </c>
       <c r="B90" s="199" t="n">
         <v>112</v>
@@ -3775,7 +3780,10 @@
       <c r="G91" s="217" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="200" t="inlineStr"/>
+      <c r="A92" s="200">
+        <f>Inquilini!B9</f>
+        <v/>
+      </c>
       <c r="B92" s="199" t="n">
         <v>1708</v>
       </c>
@@ -3802,7 +3810,10 @@
       <c r="E93" s="71" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="200" t="inlineStr"/>
+      <c r="A94" s="200">
+        <f>Inquilini!B10</f>
+        <v/>
+      </c>
       <c r="B94" s="199" t="n">
         <v>2720</v>
       </c>
@@ -3941,7 +3952,10 @@
       <c r="D102" s="71" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="200" t="inlineStr"/>
+      <c r="A103" s="200">
+        <f>Inquilini!B2</f>
+        <v/>
+      </c>
       <c r="B103" s="85">
         <f>+C3</f>
         <v/>
@@ -3968,10 +3982,9 @@
       <c r="M104" s="231" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="200" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A105" s="200">
+        <f>Inquilini!B3</f>
+        <v/>
       </c>
       <c r="B105" s="85">
         <f>+C4</f>
@@ -3999,7 +4012,10 @@
       <c r="M106" s="231" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="200" t="inlineStr"/>
+      <c r="A107" s="200">
+        <f>Inquilini!B4</f>
+        <v/>
+      </c>
       <c r="B107" s="85">
         <f>+C5</f>
         <v/>
@@ -4026,10 +4042,9 @@
       <c r="M108" s="231" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="200" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A109" s="200">
+        <f>Inquilini!B5</f>
+        <v/>
       </c>
       <c r="B109" s="85">
         <f>+C6</f>
@@ -4058,10 +4073,9 @@
       <c r="M110" s="231" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="200" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A111" s="200">
+        <f>Inquilini!B6</f>
+        <v/>
       </c>
       <c r="B111" s="85">
         <f>+C7</f>
@@ -4089,7 +4103,10 @@
       <c r="M112" s="231" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="200" t="inlineStr"/>
+      <c r="A113" s="200">
+        <f>Inquilini!B7</f>
+        <v/>
+      </c>
       <c r="B113" s="85">
         <f>+C8</f>
         <v/>
@@ -4116,10 +4133,9 @@
       <c r="M114" s="231" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="200" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A115" s="200">
+        <f>Inquilini!B8</f>
+        <v/>
       </c>
       <c r="B115" s="85">
         <f>+C9</f>
@@ -4148,7 +4164,10 @@
       <c r="M116" s="231" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="200" t="inlineStr"/>
+      <c r="A117" s="200">
+        <f>Inquilini!B9</f>
+        <v/>
+      </c>
       <c r="B117" s="85">
         <f>+C10</f>
         <v/>
@@ -4175,7 +4194,10 @@
       <c r="M118" s="231" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="200" t="inlineStr"/>
+      <c r="A119" s="200">
+        <f>Inquilini!B10</f>
+        <v/>
+      </c>
       <c r="B119" s="85">
         <f>+C11</f>
         <v/>
@@ -4345,7 +4367,10 @@
       <c r="F129" s="71" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="200" t="inlineStr"/>
+      <c r="A130" s="200">
+        <f>Inquilini!B2</f>
+        <v/>
+      </c>
       <c r="B130" s="330" t="n">
         <v>28.114</v>
       </c>
@@ -4380,10 +4405,9 @@
       <c r="H131" s="217" t="n"/>
     </row>
     <row r="132" ht="14.4" customHeight="1">
-      <c r="A132" s="200" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A132" s="200">
+        <f>Inquilini!B3</f>
+        <v/>
       </c>
       <c r="B132" s="330" t="n">
         <v>28.212</v>
@@ -4417,7 +4441,10 @@
       <c r="F133" s="71" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="200" t="inlineStr"/>
+      <c r="A134" s="200">
+        <f>Inquilini!B4</f>
+        <v/>
+      </c>
       <c r="B134" s="330" t="n">
         <v>38.014</v>
       </c>
@@ -4450,10 +4477,9 @@
       <c r="F135" s="71" t="n"/>
     </row>
     <row r="136" ht="14.4" customHeight="1">
-      <c r="A136" s="200" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A136" s="200">
+        <f>Inquilini!B5</f>
+        <v/>
       </c>
       <c r="B136" s="330" t="n">
         <v>27.352</v>
@@ -4488,10 +4514,9 @@
       <c r="H137" s="216" t="n"/>
     </row>
     <row r="138" ht="14.4" customHeight="1">
-      <c r="A138" s="200" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A138" s="200">
+        <f>Inquilini!B6</f>
+        <v/>
       </c>
       <c r="B138" s="330" t="n">
         <v>22.169</v>
@@ -4525,7 +4550,10 @@
       <c r="F139" s="71" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="200" t="inlineStr"/>
+      <c r="A140" s="200">
+        <f>Inquilini!B7</f>
+        <v/>
+      </c>
       <c r="B140" s="330" t="n">
         <v>17.497</v>
       </c>
@@ -4559,10 +4587,9 @@
       <c r="H141" s="216" t="n"/>
     </row>
     <row r="142" ht="14.4" customHeight="1">
-      <c r="A142" s="200" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A142" s="200">
+        <f>Inquilini!B8</f>
+        <v/>
       </c>
       <c r="B142" s="330" t="n">
         <v>6.683</v>
@@ -4596,7 +4623,10 @@
       <c r="F143" s="71" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="200" t="inlineStr"/>
+      <c r="A144" s="200">
+        <f>Inquilini!B9</f>
+        <v/>
+      </c>
       <c r="B144" s="330" t="n">
         <v>102.587</v>
       </c>
@@ -4629,7 +4659,10 @@
       <c r="F145" s="71" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="200" t="inlineStr"/>
+      <c r="A146" s="200">
+        <f>Inquilini!B10</f>
+        <v/>
+      </c>
       <c r="B146" s="330" t="n">
         <v>69.572</v>
       </c>
@@ -4821,7 +4854,10 @@
       <c r="D157" s="71" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="200" t="inlineStr"/>
+      <c r="A158" s="200">
+        <f>Inquilini!B2</f>
+        <v/>
+      </c>
       <c r="B158" s="85">
         <f>D3</f>
         <v/>
@@ -4846,10 +4882,9 @@
       <c r="D159" s="71" t="n"/>
     </row>
     <row r="160">
-      <c r="A160" s="200" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A160" s="200">
+        <f>Inquilini!B3</f>
+        <v/>
       </c>
       <c r="B160" s="85">
         <f>D4</f>
@@ -4875,7 +4910,10 @@
       <c r="D161" s="71" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="200" t="inlineStr"/>
+      <c r="A162" s="200">
+        <f>Inquilini!B4</f>
+        <v/>
+      </c>
       <c r="B162" s="85">
         <f>D5</f>
         <v/>
@@ -4901,10 +4939,9 @@
       <c r="D163" s="71" t="n"/>
     </row>
     <row r="164">
-      <c r="A164" s="200" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A164" s="200">
+        <f>Inquilini!B5</f>
+        <v/>
       </c>
       <c r="B164" s="85">
         <f>D6</f>
@@ -4931,10 +4968,9 @@
       <c r="D165" s="71" t="n"/>
     </row>
     <row r="166">
-      <c r="A166" s="200" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A166" s="200">
+        <f>Inquilini!B6</f>
+        <v/>
       </c>
       <c r="B166" s="85">
         <f>D7</f>
@@ -4960,7 +4996,10 @@
       <c r="D167" s="71" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" s="200" t="inlineStr"/>
+      <c r="A168" s="200">
+        <f>Inquilini!B7</f>
+        <v/>
+      </c>
       <c r="B168" s="85">
         <f>D8</f>
         <v/>
@@ -4985,10 +5024,9 @@
       <c r="D169" s="71" t="n"/>
     </row>
     <row r="170">
-      <c r="A170" s="200" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A170" s="200">
+        <f>Inquilini!B8</f>
+        <v/>
       </c>
       <c r="B170" s="85">
         <f>D9</f>
@@ -5015,7 +5053,10 @@
       <c r="D171" s="71" t="n"/>
     </row>
     <row r="172">
-      <c r="A172" s="200" t="inlineStr"/>
+      <c r="A172" s="200">
+        <f>Inquilini!B9</f>
+        <v/>
+      </c>
       <c r="B172" s="85">
         <f>D10</f>
         <v/>
@@ -5040,7 +5081,10 @@
       <c r="D173" s="71" t="n"/>
     </row>
     <row r="174" ht="13.8" customHeight="1" thickBot="1">
-      <c r="A174" s="200" t="inlineStr"/>
+      <c r="A174" s="200">
+        <f>Inquilini!B10</f>
+        <v/>
+      </c>
       <c r="B174" s="85">
         <f>D11</f>
         <v/>
@@ -5187,7 +5231,10 @@
       <c r="G181" s="82" t="n"/>
     </row>
     <row r="182">
-      <c r="A182" s="200" t="inlineStr"/>
+      <c r="A182" s="200">
+        <f>Inquilini!B2</f>
+        <v/>
+      </c>
       <c r="B182" s="330" t="n">
         <v>42.48</v>
       </c>
@@ -5220,10 +5267,9 @@
       <c r="G183" s="82" t="n"/>
     </row>
     <row r="184">
-      <c r="A184" s="200" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A184" s="200">
+        <f>Inquilini!B3</f>
+        <v/>
       </c>
       <c r="B184" s="330" t="n">
         <v>49.75</v>
@@ -5257,7 +5303,10 @@
       <c r="G185" s="82" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" s="200" t="inlineStr"/>
+      <c r="A186" s="200">
+        <f>Inquilini!B4</f>
+        <v/>
+      </c>
       <c r="B186" s="341" t="n">
         <v>67</v>
       </c>
@@ -5296,10 +5345,9 @@
       <c r="G187" s="82" t="n"/>
     </row>
     <row r="188">
-      <c r="A188" s="200" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A188" s="200">
+        <f>Inquilini!B5</f>
+        <v/>
       </c>
       <c r="B188" s="330" t="n">
         <v>36.99</v>
@@ -5333,10 +5381,9 @@
       <c r="G189" s="82" t="n"/>
     </row>
     <row r="190">
-      <c r="A190" s="200" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A190" s="200">
+        <f>Inquilini!B6</f>
+        <v/>
       </c>
       <c r="B190" s="330" t="n">
         <v>23.37</v>
@@ -5370,7 +5417,10 @@
       <c r="G191" s="82" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="200" t="inlineStr"/>
+      <c r="A192" s="200">
+        <f>Inquilini!B7</f>
+        <v/>
+      </c>
       <c r="B192" s="330" t="n">
         <v>19.67</v>
       </c>
@@ -5403,10 +5453,9 @@
       <c r="G193" s="82" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="200" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A194" s="200">
+        <f>Inquilini!B8</f>
+        <v/>
       </c>
       <c r="B194" s="330" t="n">
         <v>6.87</v>
@@ -5443,7 +5492,10 @@
       <c r="G195" s="82" t="n"/>
     </row>
     <row r="196">
-      <c r="A196" s="200" t="inlineStr"/>
+      <c r="A196" s="200">
+        <f>Inquilini!B9</f>
+        <v/>
+      </c>
       <c r="B196" s="330" t="n">
         <v>88.23999999999999</v>
       </c>
@@ -5479,7 +5531,10 @@
       <c r="G197" s="82" t="n"/>
     </row>
     <row r="198">
-      <c r="A198" s="200" t="inlineStr"/>
+      <c r="A198" s="200">
+        <f>Inquilini!B10</f>
+        <v/>
+      </c>
       <c r="B198" s="330" t="n">
         <v>51.03</v>
       </c>
@@ -5606,7 +5661,10 @@
       <c r="E204" s="80" t="n"/>
     </row>
     <row r="205">
-      <c r="A205" s="200" t="inlineStr"/>
+      <c r="A205" s="200">
+        <f>Inquilini!B2</f>
+        <v/>
+      </c>
       <c r="B205" s="279">
         <f>+C3</f>
         <v/>
@@ -5633,10 +5691,9 @@
       <c r="E206" s="80" t="n"/>
     </row>
     <row r="207">
-      <c r="A207" s="200" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A207" s="200">
+        <f>Inquilini!B3</f>
+        <v/>
       </c>
       <c r="B207" s="279">
         <f>+C4</f>
@@ -5664,7 +5721,10 @@
       <c r="E208" s="80" t="n"/>
     </row>
     <row r="209">
-      <c r="A209" s="72" t="inlineStr"/>
+      <c r="A209" s="72">
+        <f>Inquilini!B4</f>
+        <v/>
+      </c>
       <c r="B209" s="279">
         <f>+C5</f>
         <v/>
@@ -5691,10 +5751,9 @@
       <c r="E210" s="80" t="n"/>
     </row>
     <row r="211">
-      <c r="A211" s="200" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A211" s="200">
+        <f>Inquilini!B5</f>
+        <v/>
       </c>
       <c r="B211" s="279">
         <f>+C6</f>
@@ -5722,10 +5781,9 @@
       <c r="E212" s="80" t="n"/>
     </row>
     <row r="213">
-      <c r="A213" s="200" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A213" s="200">
+        <f>Inquilini!B6</f>
+        <v/>
       </c>
       <c r="B213" s="279">
         <f>+C7</f>
@@ -5753,7 +5811,10 @@
       <c r="E214" s="80" t="n"/>
     </row>
     <row r="215">
-      <c r="A215" s="200" t="inlineStr"/>
+      <c r="A215" s="200">
+        <f>Inquilini!B7</f>
+        <v/>
+      </c>
       <c r="B215" s="279">
         <f>+C8</f>
         <v/>
@@ -5780,10 +5841,9 @@
       <c r="E216" s="80" t="n"/>
     </row>
     <row r="217">
-      <c r="A217" s="200" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A217" s="200">
+        <f>Inquilini!B8</f>
+        <v/>
       </c>
       <c r="B217" s="279">
         <f>+C9</f>
@@ -5811,7 +5871,10 @@
       <c r="E218" s="80" t="n"/>
     </row>
     <row r="219">
-      <c r="A219" s="200" t="inlineStr"/>
+      <c r="A219" s="200">
+        <f>Inquilini!B9</f>
+        <v/>
+      </c>
       <c r="B219" s="279">
         <f>+C10</f>
         <v/>
@@ -5838,7 +5901,10 @@
       <c r="E220" s="80" t="n"/>
     </row>
     <row r="221">
-      <c r="A221" s="200" t="inlineStr"/>
+      <c r="A221" s="200">
+        <f>Inquilini!B10</f>
+        <v/>
+      </c>
       <c r="B221" s="279">
         <f>+C11</f>
         <v/>
@@ -6044,7 +6110,10 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="200" t="inlineStr"/>
+      <c r="A229" s="200">
+        <f>Inquilini!B2</f>
+        <v/>
+      </c>
       <c r="B229" s="126">
         <f>+F130</f>
         <v/>
@@ -6097,10 +6166,9 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="200" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A231" s="200">
+        <f>Inquilini!B3</f>
+        <v/>
       </c>
       <c r="B231" s="126">
         <f>+F132</f>
@@ -6154,7 +6222,10 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="200" t="inlineStr"/>
+      <c r="A233" s="200">
+        <f>Inquilini!B4</f>
+        <v/>
+      </c>
       <c r="B233" s="126">
         <f>+F134</f>
         <v/>
@@ -6207,10 +6278,9 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="200" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A235" s="200">
+        <f>Inquilini!B5</f>
+        <v/>
       </c>
       <c r="B235" s="126">
         <f>+F136</f>
@@ -6264,10 +6334,9 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="200" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A237" s="200">
+        <f>Inquilini!B6</f>
+        <v/>
       </c>
       <c r="B237" s="126">
         <f>+F138</f>
@@ -6321,7 +6390,10 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="200" t="inlineStr"/>
+      <c r="A239" s="200">
+        <f>Inquilini!B7</f>
+        <v/>
+      </c>
       <c r="B239" s="126">
         <f>+F140</f>
         <v/>
@@ -6374,10 +6446,9 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="200" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A241" s="200">
+        <f>Inquilini!B8</f>
+        <v/>
       </c>
       <c r="B241" s="126">
         <f>+F142</f>
@@ -6432,7 +6503,10 @@
       <c r="K242" s="56" t="n"/>
     </row>
     <row r="243">
-      <c r="A243" s="200" t="inlineStr"/>
+      <c r="A243" s="200">
+        <f>Inquilini!B9</f>
+        <v/>
+      </c>
       <c r="B243" s="126">
         <f>+F144</f>
         <v/>
@@ -6487,7 +6561,10 @@
       <c r="K244" s="56" t="n"/>
     </row>
     <row r="245">
-      <c r="A245" s="200" t="inlineStr"/>
+      <c r="A245" s="200">
+        <f>Inquilini!B10</f>
+        <v/>
+      </c>
       <c r="B245" s="126">
         <f>+F146</f>
         <v/>
@@ -6627,7 +6704,6 @@
         <v/>
       </c>
     </row>
-    <row r="249"/>
     <row r="250">
       <c r="A250" s="18" t="n"/>
       <c r="C250" s="189">
@@ -6846,7 +6922,10 @@
       <c r="P258" s="80" t="n"/>
     </row>
     <row r="259">
-      <c r="A259" s="200" t="inlineStr"/>
+      <c r="A259" s="200">
+        <f>Inquilini!B2</f>
+        <v/>
+      </c>
       <c r="B259" s="126" t="n"/>
       <c r="C259" s="127" t="n"/>
       <c r="D259" s="126" t="n"/>
@@ -6882,10 +6961,9 @@
       <c r="P260" s="80" t="n"/>
     </row>
     <row r="261" ht="14.4" customHeight="1">
-      <c r="A261" s="200" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A261" s="200">
+        <f>Inquilini!B3</f>
+        <v/>
       </c>
       <c r="B261" s="126" t="n"/>
       <c r="C261" s="127" t="n"/>
@@ -6939,7 +7017,10 @@
       <c r="P262" s="80" t="n"/>
     </row>
     <row r="263">
-      <c r="A263" s="200" t="inlineStr"/>
+      <c r="A263" s="200">
+        <f>Inquilini!B4</f>
+        <v/>
+      </c>
       <c r="B263" s="126" t="n"/>
       <c r="C263" s="127" t="n"/>
       <c r="D263" s="126" t="n"/>
@@ -6977,10 +7058,9 @@
       <c r="P264" s="80" t="n"/>
     </row>
     <row r="265" ht="14.4" customHeight="1">
-      <c r="A265" s="200" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A265" s="200">
+        <f>Inquilini!B5</f>
+        <v/>
       </c>
       <c r="B265" s="126" t="n"/>
       <c r="C265" s="127" t="n"/>
@@ -7039,10 +7119,9 @@
       <c r="P266" s="80" t="n"/>
     </row>
     <row r="267" ht="14.4" customHeight="1">
-      <c r="A267" s="200" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A267" s="200">
+        <f>Inquilini!B6</f>
+        <v/>
       </c>
       <c r="B267" s="126" t="n"/>
       <c r="C267" s="127" t="n"/>
@@ -7101,7 +7180,10 @@
       <c r="P268" s="80" t="n"/>
     </row>
     <row r="269">
-      <c r="A269" s="200" t="inlineStr"/>
+      <c r="A269" s="200">
+        <f>Inquilini!B7</f>
+        <v/>
+      </c>
       <c r="B269" s="126" t="n"/>
       <c r="C269" s="127" t="n"/>
       <c r="D269" s="126" t="n"/>
@@ -7139,10 +7221,9 @@
       <c r="P270" s="80" t="n"/>
     </row>
     <row r="271" ht="14.4" customHeight="1">
-      <c r="A271" s="200" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A271" s="200">
+        <f>Inquilini!B8</f>
+        <v/>
       </c>
       <c r="B271" s="126" t="n"/>
       <c r="C271" s="127" t="n"/>
@@ -7195,7 +7276,10 @@
       <c r="P272" s="80" t="n"/>
     </row>
     <row r="273" ht="14.4" customHeight="1">
-      <c r="A273" s="200" t="inlineStr"/>
+      <c r="A273" s="200">
+        <f>Inquilini!B9</f>
+        <v/>
+      </c>
       <c r="B273" s="126" t="n"/>
       <c r="C273" s="127" t="n"/>
       <c r="D273" s="126" t="n"/>
@@ -7242,7 +7326,10 @@
       <c r="P274" s="80" t="n"/>
     </row>
     <row r="275">
-      <c r="A275" s="200" t="inlineStr"/>
+      <c r="A275" s="200">
+        <f>Inquilini!B10</f>
+        <v/>
+      </c>
       <c r="B275" s="126" t="n"/>
       <c r="C275" s="127" t="n"/>
       <c r="D275" s="126" t="n"/>
@@ -7379,7 +7466,6 @@
       <c r="O282" s="249" t="n"/>
       <c r="P282" s="250" t="n"/>
     </row>
-    <row r="283"/>
     <row r="284">
       <c r="M284" s="235" t="n"/>
     </row>

</xml_diff>

<commit_message>
fix: all apartment labels reference Inquilini sheet, FC_report names written there only
</commit_message>
<xml_diff>
--- a/src/siemens_converter/template.xlsx
+++ b/src/siemens_converter/template.xlsx
@@ -2524,10 +2524,9 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="232" t="inlineStr">
-        <is>
-          <t>App. 01</t>
-        </is>
+      <c r="A3" s="232">
+        <f>Inquilini!A2</f>
+        <v/>
       </c>
       <c r="B3" s="9" t="n"/>
       <c r="C3" s="10">
@@ -2540,10 +2539,9 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="232" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A4" s="232">
+        <f>Inquilini!A3</f>
+        <v/>
       </c>
       <c r="B4" s="9" t="n"/>
       <c r="C4" s="10">
@@ -2556,10 +2554,9 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="232" t="inlineStr">
-        <is>
-          <t>App. 03</t>
-        </is>
+      <c r="A5" s="232">
+        <f>Inquilini!A4</f>
+        <v/>
       </c>
       <c r="B5" s="9" t="n"/>
       <c r="C5" s="10">
@@ -2572,10 +2569,9 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="232" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A6" s="232">
+        <f>Inquilini!A5</f>
+        <v/>
       </c>
       <c r="B6" s="9" t="n"/>
       <c r="C6" s="10">
@@ -2588,10 +2584,9 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="232" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A7" s="232">
+        <f>Inquilini!A6</f>
+        <v/>
       </c>
       <c r="B7" s="9" t="n"/>
       <c r="C7" s="10">
@@ -2604,10 +2599,9 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="232" t="inlineStr">
-        <is>
-          <t>App. 06</t>
-        </is>
+      <c r="A8" s="232">
+        <f>Inquilini!A7</f>
+        <v/>
       </c>
       <c r="B8" s="9" t="n"/>
       <c r="C8" s="10">
@@ -2620,10 +2614,9 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="232" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A9" s="232">
+        <f>Inquilini!A8</f>
+        <v/>
       </c>
       <c r="B9" s="9" t="n"/>
       <c r="C9" s="10">
@@ -2636,10 +2629,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="232" t="inlineStr">
-        <is>
-          <t>App. 08</t>
-        </is>
+      <c r="A10" s="232">
+        <f>Inquilini!A9</f>
+        <v/>
       </c>
       <c r="B10" s="9" t="n"/>
       <c r="C10" s="10">
@@ -2652,10 +2644,9 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="232" t="inlineStr">
-        <is>
-          <t>App. 09</t>
-        </is>
+      <c r="A11" s="232">
+        <f>Inquilini!A10</f>
+        <v/>
       </c>
       <c r="B11" s="9" t="n"/>
       <c r="C11" s="10">
@@ -2668,10 +2659,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>App. 10</t>
-        </is>
+      <c r="A12" s="8">
+        <f>Inquilini!A11</f>
+        <v/>
       </c>
       <c r="B12" s="9" t="n"/>
       <c r="C12" s="10">
@@ -3551,7 +3541,7 @@
     </row>
     <row r="77">
       <c r="A77" s="68">
-        <f>+A3</f>
+        <f>Inquilini!A2</f>
         <v/>
       </c>
       <c r="B77" s="69" t="n">
@@ -3569,7 +3559,7 @@
     </row>
     <row r="78">
       <c r="A78" s="200">
-        <f>Inquilini!B2</f>
+        <f>Inquilini!A2</f>
         <v/>
       </c>
       <c r="B78" s="199" t="n">
@@ -3589,7 +3579,7 @@
     </row>
     <row r="79">
       <c r="A79" s="68">
-        <f>+A4</f>
+        <f>Inquilini!A3</f>
         <v/>
       </c>
       <c r="B79" s="69" t="n"/>
@@ -3601,7 +3591,7 @@
     </row>
     <row r="80">
       <c r="A80" s="200">
-        <f>Inquilini!B3</f>
+        <f>Inquilini!A3</f>
         <v/>
       </c>
       <c r="B80" s="199" t="n">
@@ -3620,7 +3610,7 @@
     </row>
     <row r="81">
       <c r="A81" s="68">
-        <f>+A5</f>
+        <f>Inquilini!A4</f>
         <v/>
       </c>
       <c r="B81" s="69" t="n"/>
@@ -3631,7 +3621,7 @@
     </row>
     <row r="82">
       <c r="A82" s="200">
-        <f>Inquilini!B4</f>
+        <f>Inquilini!A4</f>
         <v/>
       </c>
       <c r="B82" s="199" t="n">
@@ -3650,7 +3640,7 @@
     </row>
     <row r="83">
       <c r="A83" s="192">
-        <f>+A6</f>
+        <f>Inquilini!A5</f>
         <v/>
       </c>
       <c r="B83" s="69" t="n"/>
@@ -3661,7 +3651,7 @@
     </row>
     <row r="84">
       <c r="A84" s="200">
-        <f>Inquilini!B5</f>
+        <f>Inquilini!A5</f>
         <v/>
       </c>
       <c r="B84" s="199" t="n">
@@ -3680,7 +3670,7 @@
     </row>
     <row r="85">
       <c r="A85" s="68">
-        <f>+A7</f>
+        <f>Inquilini!A6</f>
         <v/>
       </c>
       <c r="B85" s="69" t="n"/>
@@ -3691,7 +3681,7 @@
     </row>
     <row r="86">
       <c r="A86" s="200">
-        <f>Inquilini!B6</f>
+        <f>Inquilini!A6</f>
         <v/>
       </c>
       <c r="B86" s="199" t="n">
@@ -3710,7 +3700,7 @@
     </row>
     <row r="87">
       <c r="A87" s="68">
-        <f>+A8</f>
+        <f>Inquilini!A7</f>
         <v/>
       </c>
       <c r="B87" s="69" t="n"/>
@@ -3721,7 +3711,7 @@
     </row>
     <row r="88">
       <c r="A88" s="200">
-        <f>Inquilini!B7</f>
+        <f>Inquilini!A7</f>
         <v/>
       </c>
       <c r="B88" s="199" t="n">
@@ -3740,7 +3730,7 @@
     </row>
     <row r="89">
       <c r="A89" s="68">
-        <f>+A9</f>
+        <f>Inquilini!A8</f>
         <v/>
       </c>
       <c r="B89" s="69" t="n"/>
@@ -3751,7 +3741,7 @@
     </row>
     <row r="90">
       <c r="A90" s="200">
-        <f>Inquilini!B8</f>
+        <f>Inquilini!A8</f>
         <v/>
       </c>
       <c r="B90" s="199" t="n">
@@ -3770,7 +3760,7 @@
     </row>
     <row r="91">
       <c r="A91" s="68">
-        <f>+A10</f>
+        <f>Inquilini!A9</f>
         <v/>
       </c>
       <c r="B91" s="69" t="n"/>
@@ -3781,7 +3771,7 @@
     </row>
     <row r="92">
       <c r="A92" s="200">
-        <f>Inquilini!B9</f>
+        <f>Inquilini!A9</f>
         <v/>
       </c>
       <c r="B92" s="199" t="n">
@@ -3801,7 +3791,7 @@
     </row>
     <row r="93">
       <c r="A93" s="68">
-        <f>+A11</f>
+        <f>Inquilini!A10</f>
         <v/>
       </c>
       <c r="B93" s="69" t="n"/>
@@ -3811,7 +3801,7 @@
     </row>
     <row r="94">
       <c r="A94" s="200">
-        <f>Inquilini!B10</f>
+        <f>Inquilini!A10</f>
         <v/>
       </c>
       <c r="B94" s="199" t="n">
@@ -3831,7 +3821,7 @@
     </row>
     <row r="95" ht="13.8" customHeight="1" thickBot="1">
       <c r="A95" s="43">
-        <f>+A12</f>
+        <f>Inquilini!A11</f>
         <v/>
       </c>
       <c r="B95" s="274" t="n">
@@ -3942,10 +3932,9 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="68" t="inlineStr">
-        <is>
-          <t>App. 01</t>
-        </is>
+      <c r="A102" s="68">
+        <f>Inquilini!A2</f>
+        <v/>
       </c>
       <c r="B102" s="83" t="n"/>
       <c r="C102" s="84" t="n"/>
@@ -3953,7 +3942,7 @@
     </row>
     <row r="103">
       <c r="A103" s="200">
-        <f>Inquilini!B2</f>
+        <f>Inquilini!A2</f>
         <v/>
       </c>
       <c r="B103" s="85">
@@ -3971,10 +3960,9 @@
       <c r="M103" s="231" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="68" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A104" s="68">
+        <f>Inquilini!A3</f>
+        <v/>
       </c>
       <c r="B104" s="83" t="n"/>
       <c r="C104" s="84" t="n"/>
@@ -3983,7 +3971,7 @@
     </row>
     <row r="105">
       <c r="A105" s="200">
-        <f>Inquilini!B3</f>
+        <f>Inquilini!A3</f>
         <v/>
       </c>
       <c r="B105" s="85">
@@ -4001,10 +3989,9 @@
       <c r="M105" s="231" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="68" t="inlineStr">
-        <is>
-          <t>App. 03</t>
-        </is>
+      <c r="A106" s="68">
+        <f>Inquilini!A4</f>
+        <v/>
       </c>
       <c r="B106" s="83" t="n"/>
       <c r="C106" s="84" t="n"/>
@@ -4013,7 +4000,7 @@
     </row>
     <row r="107">
       <c r="A107" s="200">
-        <f>Inquilini!B4</f>
+        <f>Inquilini!A4</f>
         <v/>
       </c>
       <c r="B107" s="85">
@@ -4031,10 +4018,9 @@
       <c r="M107" s="231" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="192" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A108" s="192">
+        <f>Inquilini!A5</f>
+        <v/>
       </c>
       <c r="B108" s="83" t="n"/>
       <c r="C108" s="84" t="n"/>
@@ -4043,7 +4029,7 @@
     </row>
     <row r="109">
       <c r="A109" s="200">
-        <f>Inquilini!B5</f>
+        <f>Inquilini!A5</f>
         <v/>
       </c>
       <c r="B109" s="85">
@@ -4062,10 +4048,9 @@
       <c r="M109" s="231" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="192" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A110" s="192">
+        <f>Inquilini!A6</f>
+        <v/>
       </c>
       <c r="B110" s="83" t="n"/>
       <c r="C110" s="84" t="n"/>
@@ -4074,7 +4059,7 @@
     </row>
     <row r="111">
       <c r="A111" s="200">
-        <f>Inquilini!B6</f>
+        <f>Inquilini!A6</f>
         <v/>
       </c>
       <c r="B111" s="85">
@@ -4092,10 +4077,9 @@
       <c r="M111" s="231" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="68" t="inlineStr">
-        <is>
-          <t>App. 06</t>
-        </is>
+      <c r="A112" s="68">
+        <f>Inquilini!A7</f>
+        <v/>
       </c>
       <c r="B112" s="83" t="n"/>
       <c r="C112" s="84" t="n"/>
@@ -4104,7 +4088,7 @@
     </row>
     <row r="113">
       <c r="A113" s="200">
-        <f>Inquilini!B7</f>
+        <f>Inquilini!A7</f>
         <v/>
       </c>
       <c r="B113" s="85">
@@ -4122,10 +4106,9 @@
       <c r="M113" s="231" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="68" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A114" s="68">
+        <f>Inquilini!A8</f>
+        <v/>
       </c>
       <c r="B114" s="83" t="n"/>
       <c r="C114" s="84" t="n"/>
@@ -4134,7 +4117,7 @@
     </row>
     <row r="115">
       <c r="A115" s="200">
-        <f>Inquilini!B8</f>
+        <f>Inquilini!A8</f>
         <v/>
       </c>
       <c r="B115" s="85">
@@ -4153,10 +4136,9 @@
       <c r="M115" s="231" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="68" t="inlineStr">
-        <is>
-          <t>App. 08</t>
-        </is>
+      <c r="A116" s="68">
+        <f>Inquilini!A9</f>
+        <v/>
       </c>
       <c r="B116" s="83" t="n"/>
       <c r="C116" s="84" t="n"/>
@@ -4165,7 +4147,7 @@
     </row>
     <row r="117">
       <c r="A117" s="200">
-        <f>Inquilini!B9</f>
+        <f>Inquilini!A9</f>
         <v/>
       </c>
       <c r="B117" s="85">
@@ -4183,10 +4165,9 @@
       <c r="M117" s="231" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="68" t="inlineStr">
-        <is>
-          <t>App. 09</t>
-        </is>
+      <c r="A118" s="68">
+        <f>Inquilini!A10</f>
+        <v/>
       </c>
       <c r="B118" s="83" t="n"/>
       <c r="C118" s="84" t="n"/>
@@ -4195,7 +4176,7 @@
     </row>
     <row r="119">
       <c r="A119" s="200">
-        <f>Inquilini!B10</f>
+        <f>Inquilini!A10</f>
         <v/>
       </c>
       <c r="B119" s="85">
@@ -4212,10 +4193,9 @@
       </c>
     </row>
     <row r="120" ht="13.8" customHeight="1" thickBot="1">
-      <c r="A120" s="25" t="inlineStr">
-        <is>
-          <t>App. 10</t>
-        </is>
+      <c r="A120" s="25">
+        <f>Inquilini!A11</f>
+        <v/>
       </c>
       <c r="B120" s="87">
         <f>+C12</f>
@@ -4355,10 +4335,9 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="68" t="inlineStr">
-        <is>
-          <t>App. 01</t>
-        </is>
+      <c r="A129" s="68">
+        <f>Inquilini!A2</f>
+        <v/>
       </c>
       <c r="B129" s="328" t="n"/>
       <c r="C129" s="329" t="n"/>
@@ -4368,7 +4347,7 @@
     </row>
     <row r="130">
       <c r="A130" s="200">
-        <f>Inquilini!B2</f>
+        <f>Inquilini!A2</f>
         <v/>
       </c>
       <c r="B130" s="330" t="n">
@@ -4391,10 +4370,9 @@
       <c r="H130" s="217" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="68" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A131" s="68">
+        <f>Inquilini!A3</f>
+        <v/>
       </c>
       <c r="B131" s="328" t="n"/>
       <c r="C131" s="333" t="n"/>
@@ -4406,7 +4384,7 @@
     </row>
     <row r="132" ht="14.4" customHeight="1">
       <c r="A132" s="200">
-        <f>Inquilini!B3</f>
+        <f>Inquilini!A3</f>
         <v/>
       </c>
       <c r="B132" s="330" t="n">
@@ -4429,10 +4407,9 @@
       <c r="H132" s="229" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="68" t="inlineStr">
-        <is>
-          <t>App. 03</t>
-        </is>
+      <c r="A133" s="68">
+        <f>Inquilini!A4</f>
+        <v/>
       </c>
       <c r="B133" s="328" t="n"/>
       <c r="C133" s="329" t="n"/>
@@ -4442,7 +4419,7 @@
     </row>
     <row r="134">
       <c r="A134" s="200">
-        <f>Inquilini!B4</f>
+        <f>Inquilini!A4</f>
         <v/>
       </c>
       <c r="B134" s="330" t="n">
@@ -4465,10 +4442,9 @@
       <c r="H134" s="216" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="192" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A135" s="192">
+        <f>Inquilini!A5</f>
+        <v/>
       </c>
       <c r="B135" s="328" t="n"/>
       <c r="C135" s="333" t="n"/>
@@ -4478,7 +4454,7 @@
     </row>
     <row r="136" ht="14.4" customHeight="1">
       <c r="A136" s="200">
-        <f>Inquilini!B5</f>
+        <f>Inquilini!A5</f>
         <v/>
       </c>
       <c r="B136" s="330" t="n">
@@ -4501,10 +4477,9 @@
       <c r="H136" s="229" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="192" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A137" s="192">
+        <f>Inquilini!A6</f>
+        <v/>
       </c>
       <c r="B137" s="328" t="n"/>
       <c r="C137" s="333" t="n"/>
@@ -4515,7 +4490,7 @@
     </row>
     <row r="138" ht="14.4" customHeight="1">
       <c r="A138" s="200">
-        <f>Inquilini!B6</f>
+        <f>Inquilini!A6</f>
         <v/>
       </c>
       <c r="B138" s="330" t="n">
@@ -4538,10 +4513,9 @@
       <c r="H138" s="229" t="n"/>
     </row>
     <row r="139">
-      <c r="A139" s="68" t="inlineStr">
-        <is>
-          <t>App. 06</t>
-        </is>
+      <c r="A139" s="68">
+        <f>Inquilini!A7</f>
+        <v/>
       </c>
       <c r="B139" s="328" t="n"/>
       <c r="C139" s="329" t="n"/>
@@ -4551,7 +4525,7 @@
     </row>
     <row r="140">
       <c r="A140" s="200">
-        <f>Inquilini!B7</f>
+        <f>Inquilini!A7</f>
         <v/>
       </c>
       <c r="B140" s="330" t="n">
@@ -4574,10 +4548,9 @@
       <c r="H140" s="216" t="n"/>
     </row>
     <row r="141">
-      <c r="A141" s="68" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A141" s="68">
+        <f>Inquilini!A8</f>
+        <v/>
       </c>
       <c r="B141" s="328" t="n"/>
       <c r="C141" s="334" t="n"/>
@@ -4588,7 +4561,7 @@
     </row>
     <row r="142" ht="14.4" customHeight="1">
       <c r="A142" s="200">
-        <f>Inquilini!B8</f>
+        <f>Inquilini!A8</f>
         <v/>
       </c>
       <c r="B142" s="330" t="n">
@@ -4611,10 +4584,9 @@
       <c r="H142" s="229" t="n"/>
     </row>
     <row r="143">
-      <c r="A143" s="68" t="inlineStr">
-        <is>
-          <t>App. 08</t>
-        </is>
+      <c r="A143" s="68">
+        <f>Inquilini!A9</f>
+        <v/>
       </c>
       <c r="B143" s="328" t="n"/>
       <c r="C143" s="329" t="n"/>
@@ -4624,7 +4596,7 @@
     </row>
     <row r="144">
       <c r="A144" s="200">
-        <f>Inquilini!B9</f>
+        <f>Inquilini!A9</f>
         <v/>
       </c>
       <c r="B144" s="330" t="n">
@@ -4647,10 +4619,9 @@
       <c r="H144" s="217" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="68" t="inlineStr">
-        <is>
-          <t>App. 09</t>
-        </is>
+      <c r="A145" s="68">
+        <f>Inquilini!A10</f>
+        <v/>
       </c>
       <c r="B145" s="328" t="n"/>
       <c r="C145" s="329" t="n"/>
@@ -4660,7 +4631,7 @@
     </row>
     <row r="146">
       <c r="A146" s="200">
-        <f>Inquilini!B10</f>
+        <f>Inquilini!A10</f>
         <v/>
       </c>
       <c r="B146" s="330" t="n">
@@ -4683,10 +4654,9 @@
       <c r="H146" s="217" t="n"/>
     </row>
     <row r="147" ht="13.8" customHeight="1" thickBot="1">
-      <c r="A147" s="25" t="inlineStr">
-        <is>
-          <t>App. 10</t>
-        </is>
+      <c r="A147" s="25">
+        <f>Inquilini!A11</f>
+        <v/>
       </c>
       <c r="B147" s="335" t="n">
         <v>73.76000000000001</v>
@@ -4844,10 +4814,9 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="68" t="inlineStr">
-        <is>
-          <t>App. 01</t>
-        </is>
+      <c r="A157" s="68">
+        <f>Inquilini!A2</f>
+        <v/>
       </c>
       <c r="B157" s="83" t="n"/>
       <c r="C157" s="70" t="n"/>
@@ -4855,7 +4824,7 @@
     </row>
     <row r="158">
       <c r="A158" s="200">
-        <f>Inquilini!B2</f>
+        <f>Inquilini!A2</f>
         <v/>
       </c>
       <c r="B158" s="85">
@@ -4872,10 +4841,9 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="68" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A159" s="68">
+        <f>Inquilini!A3</f>
+        <v/>
       </c>
       <c r="B159" s="83" t="n"/>
       <c r="C159" s="70" t="n"/>
@@ -4883,7 +4851,7 @@
     </row>
     <row r="160">
       <c r="A160" s="200">
-        <f>Inquilini!B3</f>
+        <f>Inquilini!A3</f>
         <v/>
       </c>
       <c r="B160" s="85">
@@ -4900,10 +4868,9 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="68" t="inlineStr">
-        <is>
-          <t>App. 03</t>
-        </is>
+      <c r="A161" s="68">
+        <f>Inquilini!A4</f>
+        <v/>
       </c>
       <c r="B161" s="83" t="n"/>
       <c r="C161" s="70" t="n"/>
@@ -4911,7 +4878,7 @@
     </row>
     <row r="162">
       <c r="A162" s="200">
-        <f>Inquilini!B4</f>
+        <f>Inquilini!A4</f>
         <v/>
       </c>
       <c r="B162" s="85">
@@ -4929,10 +4896,9 @@
       <c r="E162" s="231" t="n"/>
     </row>
     <row r="163">
-      <c r="A163" s="192" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A163" s="192">
+        <f>Inquilini!A5</f>
+        <v/>
       </c>
       <c r="B163" s="83" t="n"/>
       <c r="C163" s="70" t="n"/>
@@ -4940,7 +4906,7 @@
     </row>
     <row r="164">
       <c r="A164" s="200">
-        <f>Inquilini!B5</f>
+        <f>Inquilini!A5</f>
         <v/>
       </c>
       <c r="B164" s="85">
@@ -4958,10 +4924,9 @@
       <c r="E164" s="18" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" s="192" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A165" s="192">
+        <f>Inquilini!A6</f>
+        <v/>
       </c>
       <c r="B165" s="83" t="n"/>
       <c r="C165" s="70" t="n"/>
@@ -4969,7 +4934,7 @@
     </row>
     <row r="166">
       <c r="A166" s="200">
-        <f>Inquilini!B6</f>
+        <f>Inquilini!A6</f>
         <v/>
       </c>
       <c r="B166" s="85">
@@ -4986,10 +4951,9 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="68" t="inlineStr">
-        <is>
-          <t>App. 06</t>
-        </is>
+      <c r="A167" s="68">
+        <f>Inquilini!A7</f>
+        <v/>
       </c>
       <c r="B167" s="83" t="n"/>
       <c r="C167" s="70" t="n"/>
@@ -4997,7 +4961,7 @@
     </row>
     <row r="168">
       <c r="A168" s="200">
-        <f>Inquilini!B7</f>
+        <f>Inquilini!A7</f>
         <v/>
       </c>
       <c r="B168" s="85">
@@ -5014,10 +4978,9 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="68" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A169" s="68">
+        <f>Inquilini!A8</f>
+        <v/>
       </c>
       <c r="B169" s="83" t="n"/>
       <c r="C169" s="70" t="n"/>
@@ -5025,7 +4988,7 @@
     </row>
     <row r="170">
       <c r="A170" s="200">
-        <f>Inquilini!B8</f>
+        <f>Inquilini!A8</f>
         <v/>
       </c>
       <c r="B170" s="85">
@@ -5043,10 +5006,9 @@
       <c r="E170" s="18" t="n"/>
     </row>
     <row r="171">
-      <c r="A171" s="68" t="inlineStr">
-        <is>
-          <t>App. 08</t>
-        </is>
+      <c r="A171" s="68">
+        <f>Inquilini!A9</f>
+        <v/>
       </c>
       <c r="B171" s="83" t="n"/>
       <c r="C171" s="70" t="n"/>
@@ -5054,7 +5016,7 @@
     </row>
     <row r="172">
       <c r="A172" s="200">
-        <f>Inquilini!B9</f>
+        <f>Inquilini!A9</f>
         <v/>
       </c>
       <c r="B172" s="85">
@@ -5071,10 +5033,9 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="68" t="inlineStr">
-        <is>
-          <t>App. 09</t>
-        </is>
+      <c r="A173" s="68">
+        <f>Inquilini!A10</f>
+        <v/>
       </c>
       <c r="B173" s="83" t="n"/>
       <c r="C173" s="70" t="n"/>
@@ -5082,7 +5043,7 @@
     </row>
     <row r="174" ht="13.8" customHeight="1" thickBot="1">
       <c r="A174" s="200">
-        <f>Inquilini!B10</f>
+        <f>Inquilini!A10</f>
         <v/>
       </c>
       <c r="B174" s="85">
@@ -5099,10 +5060,9 @@
       </c>
     </row>
     <row r="175" ht="13.8" customHeight="1" thickBot="1">
-      <c r="A175" s="25" t="inlineStr">
-        <is>
-          <t>App. 10</t>
-        </is>
+      <c r="A175" s="25">
+        <f>Inquilini!A11</f>
+        <v/>
       </c>
       <c r="B175" s="87">
         <f>+D12</f>
@@ -5218,10 +5178,9 @@
       <c r="G180" s="82" t="n"/>
     </row>
     <row r="181">
-      <c r="A181" s="68" t="inlineStr">
-        <is>
-          <t>App. 01</t>
-        </is>
+      <c r="A181" s="68">
+        <f>Inquilini!A2</f>
+        <v/>
       </c>
       <c r="B181" s="328" t="n"/>
       <c r="C181" s="328" t="n"/>
@@ -5232,7 +5191,7 @@
     </row>
     <row r="182">
       <c r="A182" s="200">
-        <f>Inquilini!B2</f>
+        <f>Inquilini!A2</f>
         <v/>
       </c>
       <c r="B182" s="330" t="n">
@@ -5254,10 +5213,9 @@
       <c r="G182" s="82" t="n"/>
     </row>
     <row r="183">
-      <c r="A183" s="68" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A183" s="68">
+        <f>Inquilini!A3</f>
+        <v/>
       </c>
       <c r="B183" s="328" t="n"/>
       <c r="C183" s="328" t="n"/>
@@ -5268,7 +5226,7 @@
     </row>
     <row r="184">
       <c r="A184" s="200">
-        <f>Inquilini!B3</f>
+        <f>Inquilini!A3</f>
         <v/>
       </c>
       <c r="B184" s="330" t="n">
@@ -5290,10 +5248,9 @@
       <c r="G184" s="82" t="n"/>
     </row>
     <row r="185">
-      <c r="A185" s="68" t="inlineStr">
-        <is>
-          <t>App. 03</t>
-        </is>
+      <c r="A185" s="68">
+        <f>Inquilini!A4</f>
+        <v/>
       </c>
       <c r="B185" s="328" t="n"/>
       <c r="C185" s="328" t="n"/>
@@ -5304,7 +5261,7 @@
     </row>
     <row r="186">
       <c r="A186" s="200">
-        <f>Inquilini!B4</f>
+        <f>Inquilini!A4</f>
         <v/>
       </c>
       <c r="B186" s="341" t="n">
@@ -5332,10 +5289,9 @@
       <c r="J186" s="81" t="n"/>
     </row>
     <row r="187">
-      <c r="A187" s="190" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A187" s="190">
+        <f>Inquilini!A5</f>
+        <v/>
       </c>
       <c r="B187" s="328" t="n"/>
       <c r="C187" s="328" t="n"/>
@@ -5346,7 +5302,7 @@
     </row>
     <row r="188">
       <c r="A188" s="200">
-        <f>Inquilini!B5</f>
+        <f>Inquilini!A5</f>
         <v/>
       </c>
       <c r="B188" s="330" t="n">
@@ -5368,10 +5324,9 @@
       <c r="G188" s="82" t="n"/>
     </row>
     <row r="189">
-      <c r="A189" s="192" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A189" s="192">
+        <f>Inquilini!A6</f>
+        <v/>
       </c>
       <c r="B189" s="328" t="n"/>
       <c r="C189" s="328" t="n"/>
@@ -5382,7 +5337,7 @@
     </row>
     <row r="190">
       <c r="A190" s="200">
-        <f>Inquilini!B6</f>
+        <f>Inquilini!A6</f>
         <v/>
       </c>
       <c r="B190" s="330" t="n">
@@ -5404,10 +5359,9 @@
       <c r="G190" s="82" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" s="68" t="inlineStr">
-        <is>
-          <t>App. 06</t>
-        </is>
+      <c r="A191" s="68">
+        <f>Inquilini!A7</f>
+        <v/>
       </c>
       <c r="B191" s="328" t="n"/>
       <c r="C191" s="328" t="n"/>
@@ -5418,7 +5372,7 @@
     </row>
     <row r="192">
       <c r="A192" s="200">
-        <f>Inquilini!B7</f>
+        <f>Inquilini!A7</f>
         <v/>
       </c>
       <c r="B192" s="330" t="n">
@@ -5440,10 +5394,9 @@
       <c r="G192" s="82" t="n"/>
     </row>
     <row r="193">
-      <c r="A193" s="68" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A193" s="68">
+        <f>Inquilini!A8</f>
+        <v/>
       </c>
       <c r="B193" s="328" t="n"/>
       <c r="C193" s="328" t="n"/>
@@ -5454,7 +5407,7 @@
     </row>
     <row r="194">
       <c r="A194" s="200">
-        <f>Inquilini!B8</f>
+        <f>Inquilini!A8</f>
         <v/>
       </c>
       <c r="B194" s="330" t="n">
@@ -5476,10 +5429,9 @@
       <c r="G194" s="82" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" s="68" t="inlineStr">
-        <is>
-          <t>App. 08</t>
-        </is>
+      <c r="A195" s="68">
+        <f>Inquilini!A9</f>
+        <v/>
       </c>
       <c r="B195" s="328" t="n"/>
       <c r="C195" s="328" t="n"/>
@@ -5493,7 +5445,7 @@
     </row>
     <row r="196">
       <c r="A196" s="200">
-        <f>Inquilini!B9</f>
+        <f>Inquilini!A9</f>
         <v/>
       </c>
       <c r="B196" s="330" t="n">
@@ -5515,10 +5467,9 @@
       <c r="G196" s="82" t="n"/>
     </row>
     <row r="197">
-      <c r="A197" s="68" t="inlineStr">
-        <is>
-          <t>App. 09</t>
-        </is>
+      <c r="A197" s="68">
+        <f>Inquilini!A10</f>
+        <v/>
       </c>
       <c r="B197" s="328" t="n"/>
       <c r="C197" s="328" t="n"/>
@@ -5532,7 +5483,7 @@
     </row>
     <row r="198">
       <c r="A198" s="200">
-        <f>Inquilini!B10</f>
+        <f>Inquilini!A10</f>
         <v/>
       </c>
       <c r="B198" s="330" t="n">
@@ -5554,10 +5505,9 @@
       <c r="G198" s="82" t="n"/>
     </row>
     <row r="199" ht="13.8" customHeight="1" thickBot="1">
-      <c r="A199" s="25" t="inlineStr">
-        <is>
-          <t>App. 10</t>
-        </is>
+      <c r="A199" s="25">
+        <f>Inquilini!A11</f>
+        <v/>
       </c>
       <c r="B199" s="335" t="n">
         <v>44.23</v>
@@ -5653,16 +5603,15 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="68" t="inlineStr">
-        <is>
-          <t>App. 01</t>
-        </is>
+      <c r="A204" s="68">
+        <f>Inquilini!A2</f>
+        <v/>
       </c>
       <c r="E204" s="80" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="200">
-        <f>Inquilini!B2</f>
+        <f>Inquilini!A2</f>
         <v/>
       </c>
       <c r="B205" s="279">
@@ -5683,16 +5632,15 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="68" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A206" s="68">
+        <f>Inquilini!A3</f>
+        <v/>
       </c>
       <c r="E206" s="80" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="200">
-        <f>Inquilini!B3</f>
+        <f>Inquilini!A3</f>
         <v/>
       </c>
       <c r="B207" s="279">
@@ -5713,16 +5661,15 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="68" t="inlineStr">
-        <is>
-          <t>App. 03</t>
-        </is>
+      <c r="A208" s="68">
+        <f>Inquilini!A4</f>
+        <v/>
       </c>
       <c r="E208" s="80" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="72">
-        <f>Inquilini!B4</f>
+        <f>Inquilini!A4</f>
         <v/>
       </c>
       <c r="B209" s="279">
@@ -5743,16 +5690,15 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="192" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A210" s="192">
+        <f>Inquilini!A5</f>
+        <v/>
       </c>
       <c r="E210" s="80" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="200">
-        <f>Inquilini!B5</f>
+        <f>Inquilini!A5</f>
         <v/>
       </c>
       <c r="B211" s="279">
@@ -5773,16 +5719,15 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="192" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A212" s="192">
+        <f>Inquilini!A6</f>
+        <v/>
       </c>
       <c r="E212" s="80" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="200">
-        <f>Inquilini!B6</f>
+        <f>Inquilini!A6</f>
         <v/>
       </c>
       <c r="B213" s="279">
@@ -5803,16 +5748,15 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="68" t="inlineStr">
-        <is>
-          <t>App. 06</t>
-        </is>
+      <c r="A214" s="68">
+        <f>Inquilini!A7</f>
+        <v/>
       </c>
       <c r="E214" s="80" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="200">
-        <f>Inquilini!B7</f>
+        <f>Inquilini!A7</f>
         <v/>
       </c>
       <c r="B215" s="279">
@@ -5833,16 +5777,15 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="68" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A216" s="68">
+        <f>Inquilini!A8</f>
+        <v/>
       </c>
       <c r="E216" s="80" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="200">
-        <f>Inquilini!B8</f>
+        <f>Inquilini!A8</f>
         <v/>
       </c>
       <c r="B217" s="279">
@@ -5863,16 +5806,15 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="68" t="inlineStr">
-        <is>
-          <t>App. 08</t>
-        </is>
+      <c r="A218" s="68">
+        <f>Inquilini!A9</f>
+        <v/>
       </c>
       <c r="E218" s="80" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="200">
-        <f>Inquilini!B9</f>
+        <f>Inquilini!A9</f>
         <v/>
       </c>
       <c r="B219" s="279">
@@ -5893,16 +5835,15 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="68" t="inlineStr">
-        <is>
-          <t>App. 09</t>
-        </is>
+      <c r="A220" s="68">
+        <f>Inquilini!A10</f>
+        <v/>
       </c>
       <c r="E220" s="80" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="200">
-        <f>Inquilini!B10</f>
+        <f>Inquilini!A10</f>
         <v/>
       </c>
       <c r="B221" s="279">
@@ -5923,10 +5864,9 @@
       </c>
     </row>
     <row r="222" ht="13.8" customHeight="1" thickBot="1">
-      <c r="A222" s="25" t="inlineStr">
-        <is>
-          <t>App. 10</t>
-        </is>
+      <c r="A222" s="25">
+        <f>Inquilini!A11</f>
+        <v/>
       </c>
       <c r="B222" s="277">
         <f>+C12</f>
@@ -6092,10 +6032,9 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="68" t="inlineStr">
-        <is>
-          <t>App. 01</t>
-        </is>
+      <c r="A228" s="68">
+        <f>Inquilini!A2</f>
+        <v/>
       </c>
       <c r="B228" s="123" t="n"/>
       <c r="C228" s="124" t="n"/>
@@ -6111,7 +6050,7 @@
     </row>
     <row r="229">
       <c r="A229" s="200">
-        <f>Inquilini!B2</f>
+        <f>Inquilini!A2</f>
         <v/>
       </c>
       <c r="B229" s="126">
@@ -6148,10 +6087,9 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="68" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A230" s="68">
+        <f>Inquilini!A3</f>
+        <v/>
       </c>
       <c r="B230" s="123" t="n"/>
       <c r="C230" s="124" t="n"/>
@@ -6167,7 +6105,7 @@
     </row>
     <row r="231">
       <c r="A231" s="200">
-        <f>Inquilini!B3</f>
+        <f>Inquilini!A3</f>
         <v/>
       </c>
       <c r="B231" s="126">
@@ -6204,10 +6142,9 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="68" t="inlineStr">
-        <is>
-          <t>App. 03</t>
-        </is>
+      <c r="A232" s="68">
+        <f>Inquilini!A4</f>
+        <v/>
       </c>
       <c r="B232" s="123" t="n"/>
       <c r="C232" s="124" t="n"/>
@@ -6223,7 +6160,7 @@
     </row>
     <row r="233">
       <c r="A233" s="200">
-        <f>Inquilini!B4</f>
+        <f>Inquilini!A4</f>
         <v/>
       </c>
       <c r="B233" s="126">
@@ -6260,10 +6197,9 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="68" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A234" s="68">
+        <f>Inquilini!A5</f>
+        <v/>
       </c>
       <c r="B234" s="123" t="n"/>
       <c r="C234" s="124" t="n"/>
@@ -6279,7 +6215,7 @@
     </row>
     <row r="235">
       <c r="A235" s="200">
-        <f>Inquilini!B5</f>
+        <f>Inquilini!A5</f>
         <v/>
       </c>
       <c r="B235" s="126">
@@ -6316,10 +6252,9 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="192" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A236" s="192">
+        <f>Inquilini!A6</f>
+        <v/>
       </c>
       <c r="B236" s="123" t="n"/>
       <c r="C236" s="124" t="n"/>
@@ -6335,7 +6270,7 @@
     </row>
     <row r="237">
       <c r="A237" s="200">
-        <f>Inquilini!B6</f>
+        <f>Inquilini!A6</f>
         <v/>
       </c>
       <c r="B237" s="126">
@@ -6372,10 +6307,9 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="68" t="inlineStr">
-        <is>
-          <t>App. 06</t>
-        </is>
+      <c r="A238" s="68">
+        <f>Inquilini!A7</f>
+        <v/>
       </c>
       <c r="B238" s="123" t="n"/>
       <c r="C238" s="124" t="n"/>
@@ -6391,7 +6325,7 @@
     </row>
     <row r="239">
       <c r="A239" s="200">
-        <f>Inquilini!B7</f>
+        <f>Inquilini!A7</f>
         <v/>
       </c>
       <c r="B239" s="126">
@@ -6428,10 +6362,9 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="68" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A240" s="68">
+        <f>Inquilini!A8</f>
+        <v/>
       </c>
       <c r="B240" s="123" t="n"/>
       <c r="C240" s="124" t="n"/>
@@ -6447,7 +6380,7 @@
     </row>
     <row r="241">
       <c r="A241" s="200">
-        <f>Inquilini!B8</f>
+        <f>Inquilini!A8</f>
         <v/>
       </c>
       <c r="B241" s="126">
@@ -6484,10 +6417,9 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="68" t="inlineStr">
-        <is>
-          <t>App. 08</t>
-        </is>
+      <c r="A242" s="68">
+        <f>Inquilini!A9</f>
+        <v/>
       </c>
       <c r="B242" s="123" t="n"/>
       <c r="C242" s="124" t="n"/>
@@ -6504,7 +6436,7 @@
     </row>
     <row r="243">
       <c r="A243" s="200">
-        <f>Inquilini!B9</f>
+        <f>Inquilini!A9</f>
         <v/>
       </c>
       <c r="B243" s="126">
@@ -6542,10 +6474,9 @@
       <c r="K243" s="56" t="n"/>
     </row>
     <row r="244">
-      <c r="A244" s="68" t="inlineStr">
-        <is>
-          <t>App. 09</t>
-        </is>
+      <c r="A244" s="68">
+        <f>Inquilini!A10</f>
+        <v/>
       </c>
       <c r="B244" s="123" t="n"/>
       <c r="C244" s="124" t="n"/>
@@ -6562,7 +6493,7 @@
     </row>
     <row r="245">
       <c r="A245" s="200">
-        <f>Inquilini!B10</f>
+        <f>Inquilini!A10</f>
         <v/>
       </c>
       <c r="B245" s="126">
@@ -6600,10 +6531,9 @@
       <c r="K245" s="56" t="n"/>
     </row>
     <row r="246" ht="13.8" customHeight="1" thickBot="1">
-      <c r="A246" s="25" t="inlineStr">
-        <is>
-          <t>App. 10</t>
-        </is>
+      <c r="A246" s="25">
+        <f>Inquilini!A11</f>
+        <v/>
       </c>
       <c r="B246" s="129">
         <f>+F147</f>
@@ -6903,10 +6833,9 @@
       <c r="P257" s="80" t="n"/>
     </row>
     <row r="258">
-      <c r="A258" s="68" t="inlineStr">
-        <is>
-          <t>App. 01</t>
-        </is>
+      <c r="A258" s="68">
+        <f>Inquilini!A2</f>
+        <v/>
       </c>
       <c r="B258" s="123" t="n"/>
       <c r="C258" s="124" t="n"/>
@@ -6923,7 +6852,7 @@
     </row>
     <row r="259">
       <c r="A259" s="200">
-        <f>Inquilini!B2</f>
+        <f>Inquilini!A2</f>
         <v/>
       </c>
       <c r="B259" s="126" t="n"/>
@@ -6941,10 +6870,9 @@
       <c r="P259" s="80" t="n"/>
     </row>
     <row r="260">
-      <c r="A260" s="68" t="inlineStr">
-        <is>
-          <t>App. 02</t>
-        </is>
+      <c r="A260" s="68">
+        <f>Inquilini!A3</f>
+        <v/>
       </c>
       <c r="B260" s="123" t="n"/>
       <c r="C260" s="124" t="n"/>
@@ -6962,7 +6890,7 @@
     </row>
     <row r="261" ht="14.4" customHeight="1">
       <c r="A261" s="200">
-        <f>Inquilini!B3</f>
+        <f>Inquilini!A3</f>
         <v/>
       </c>
       <c r="B261" s="126" t="n"/>
@@ -6996,10 +6924,9 @@
       <c r="P261" s="80" t="n"/>
     </row>
     <row r="262">
-      <c r="A262" s="68" t="inlineStr">
-        <is>
-          <t>App. 03</t>
-        </is>
+      <c r="A262" s="68">
+        <f>Inquilini!A4</f>
+        <v/>
       </c>
       <c r="B262" s="123" t="n"/>
       <c r="C262" s="124" t="n"/>
@@ -7018,7 +6945,7 @@
     </row>
     <row r="263">
       <c r="A263" s="200">
-        <f>Inquilini!B4</f>
+        <f>Inquilini!A4</f>
         <v/>
       </c>
       <c r="B263" s="126" t="n"/>
@@ -7037,10 +6964,9 @@
       <c r="P263" s="80" t="n"/>
     </row>
     <row r="264">
-      <c r="A264" s="68" t="inlineStr">
-        <is>
-          <t>App. 04</t>
-        </is>
+      <c r="A264" s="68">
+        <f>Inquilini!A5</f>
+        <v/>
       </c>
       <c r="B264" s="123" t="n"/>
       <c r="C264" s="124" t="n"/>
@@ -7059,7 +6985,7 @@
     </row>
     <row r="265" ht="14.4" customHeight="1">
       <c r="A265" s="200">
-        <f>Inquilini!B5</f>
+        <f>Inquilini!A5</f>
         <v/>
       </c>
       <c r="B265" s="126" t="n"/>
@@ -7093,10 +7019,9 @@
       <c r="P265" s="80" t="n"/>
     </row>
     <row r="266">
-      <c r="A266" s="192" t="inlineStr">
-        <is>
-          <t>App. 05</t>
-        </is>
+      <c r="A266" s="192">
+        <f>Inquilini!A6</f>
+        <v/>
       </c>
       <c r="B266" s="123" t="n"/>
       <c r="C266" s="124" t="n"/>
@@ -7120,7 +7045,7 @@
     </row>
     <row r="267" ht="14.4" customHeight="1">
       <c r="A267" s="200">
-        <f>Inquilini!B6</f>
+        <f>Inquilini!A6</f>
         <v/>
       </c>
       <c r="B267" s="126" t="n"/>
@@ -7159,10 +7084,9 @@
       <c r="P267" s="80" t="n"/>
     </row>
     <row r="268">
-      <c r="A268" s="68" t="inlineStr">
-        <is>
-          <t>App. 06</t>
-        </is>
+      <c r="A268" s="68">
+        <f>Inquilini!A7</f>
+        <v/>
       </c>
       <c r="B268" s="123" t="n"/>
       <c r="C268" s="124" t="n"/>
@@ -7181,7 +7105,7 @@
     </row>
     <row r="269">
       <c r="A269" s="200">
-        <f>Inquilini!B7</f>
+        <f>Inquilini!A7</f>
         <v/>
       </c>
       <c r="B269" s="126" t="n"/>
@@ -7200,10 +7124,9 @@
       <c r="P269" s="80" t="n"/>
     </row>
     <row r="270">
-      <c r="A270" s="68" t="inlineStr">
-        <is>
-          <t>App. 07</t>
-        </is>
+      <c r="A270" s="68">
+        <f>Inquilini!A8</f>
+        <v/>
       </c>
       <c r="B270" s="123" t="n"/>
       <c r="C270" s="124" t="n"/>
@@ -7222,7 +7145,7 @@
     </row>
     <row r="271" ht="14.4" customHeight="1">
       <c r="A271" s="200">
-        <f>Inquilini!B8</f>
+        <f>Inquilini!A8</f>
         <v/>
       </c>
       <c r="B271" s="126" t="n"/>
@@ -7256,10 +7179,9 @@
       <c r="P271" s="80" t="n"/>
     </row>
     <row r="272">
-      <c r="A272" s="68" t="inlineStr">
-        <is>
-          <t>App. 08</t>
-        </is>
+      <c r="A272" s="68">
+        <f>Inquilini!A9</f>
+        <v/>
       </c>
       <c r="B272" s="123" t="n"/>
       <c r="C272" s="124" t="n"/>
@@ -7277,7 +7199,7 @@
     </row>
     <row r="273" ht="14.4" customHeight="1">
       <c r="A273" s="200">
-        <f>Inquilini!B9</f>
+        <f>Inquilini!A9</f>
         <v/>
       </c>
       <c r="B273" s="126" t="n"/>
@@ -7306,10 +7228,9 @@
       <c r="P273" s="80" t="n"/>
     </row>
     <row r="274">
-      <c r="A274" s="68" t="inlineStr">
-        <is>
-          <t>App. 09</t>
-        </is>
+      <c r="A274" s="68">
+        <f>Inquilini!A10</f>
+        <v/>
       </c>
       <c r="B274" s="123" t="n"/>
       <c r="C274" s="124" t="n"/>
@@ -7327,7 +7248,7 @@
     </row>
     <row r="275">
       <c r="A275" s="200">
-        <f>Inquilini!B10</f>
+        <f>Inquilini!A10</f>
         <v/>
       </c>
       <c r="B275" s="126" t="n"/>
@@ -7345,10 +7266,9 @@
       <c r="P275" s="80" t="n"/>
     </row>
     <row r="276" ht="13.8" customHeight="1" thickBot="1">
-      <c r="A276" s="25" t="inlineStr">
-        <is>
-          <t>App. 10</t>
-        </is>
+      <c r="A276" s="25">
+        <f>Inquilini!A11</f>
+        <v/>
       </c>
       <c r="B276" s="129" t="n"/>
       <c r="C276" s="130" t="n"/>
@@ -7991,7 +7911,10 @@
       </c>
     </row>
     <row r="4" ht="13.8" customHeight="1">
-      <c r="A4" s="166" t="n"/>
+      <c r="A4" s="166">
+        <f>Inquilini!A2</f>
+        <v/>
+      </c>
       <c r="B4" s="167" t="n"/>
       <c r="C4" s="168" t="n"/>
       <c r="D4" s="169">
@@ -8005,7 +7928,10 @@
       </c>
     </row>
     <row r="5" ht="13.8" customHeight="1">
-      <c r="A5" s="171" t="n"/>
+      <c r="A5" s="171">
+        <f>Inquilini!A3</f>
+        <v/>
+      </c>
       <c r="B5" s="167" t="n"/>
       <c r="C5" s="170" t="n"/>
       <c r="D5" s="169">
@@ -8019,7 +7945,10 @@
       </c>
     </row>
     <row r="6" ht="13.8" customHeight="1">
-      <c r="A6" s="166" t="n"/>
+      <c r="A6" s="166">
+        <f>Inquilini!A4</f>
+        <v/>
+      </c>
       <c r="B6" s="167" t="n"/>
       <c r="C6" s="170" t="n"/>
       <c r="D6" s="169">
@@ -8033,7 +7962,10 @@
       </c>
     </row>
     <row r="7" ht="13.8" customHeight="1">
-      <c r="A7" s="171" t="n"/>
+      <c r="A7" s="171">
+        <f>Inquilini!A5</f>
+        <v/>
+      </c>
       <c r="B7" s="167" t="n"/>
       <c r="C7" s="170" t="n"/>
       <c r="D7" s="169">
@@ -8047,7 +7979,10 @@
       </c>
     </row>
     <row r="8" ht="13.8" customHeight="1">
-      <c r="A8" s="171" t="n"/>
+      <c r="A8" s="171">
+        <f>Inquilini!A6</f>
+        <v/>
+      </c>
       <c r="B8" s="167" t="n"/>
       <c r="C8" s="170" t="n"/>
       <c r="D8" s="169">
@@ -8061,7 +7996,10 @@
       </c>
     </row>
     <row r="9" ht="13.8" customHeight="1">
-      <c r="A9" s="166" t="n"/>
+      <c r="A9" s="166">
+        <f>Inquilini!A7</f>
+        <v/>
+      </c>
       <c r="B9" s="167" t="n"/>
       <c r="C9" s="170" t="n"/>
       <c r="D9" s="169">
@@ -8075,7 +8013,10 @@
       </c>
     </row>
     <row r="10" ht="13.8" customHeight="1">
-      <c r="A10" s="171" t="n"/>
+      <c r="A10" s="171">
+        <f>Inquilini!A8</f>
+        <v/>
+      </c>
       <c r="B10" s="167" t="n"/>
       <c r="C10" s="170" t="n"/>
       <c r="D10" s="169">
@@ -8089,7 +8030,10 @@
       </c>
     </row>
     <row r="11" ht="13.8" customHeight="1">
-      <c r="A11" s="166" t="n"/>
+      <c r="A11" s="166">
+        <f>Inquilini!A9</f>
+        <v/>
+      </c>
       <c r="B11" s="167" t="n"/>
       <c r="C11" s="170" t="n"/>
       <c r="D11" s="169">
@@ -8103,7 +8047,10 @@
       </c>
     </row>
     <row r="12" ht="13.8" customHeight="1">
-      <c r="A12" s="166" t="n"/>
+      <c r="A12" s="166">
+        <f>Inquilini!A10</f>
+        <v/>
+      </c>
       <c r="B12" s="167" t="n"/>
       <c r="C12" s="170" t="n"/>
       <c r="D12" s="169">
@@ -8117,7 +8064,10 @@
       </c>
     </row>
     <row r="13" ht="13.8" customHeight="1">
-      <c r="A13" s="171" t="n"/>
+      <c r="A13" s="171">
+        <f>Inquilini!A11</f>
+        <v/>
+      </c>
       <c r="B13" s="167" t="n"/>
       <c r="C13" s="170" t="n"/>
       <c r="D13" s="169">

</xml_diff>

<commit_message>
fix: owner rows reference Inquilini!A, tenant rows reference Inquilini!B
</commit_message>
<xml_diff>
--- a/src/siemens_converter/template.xlsx
+++ b/src/siemens_converter/template.xlsx
@@ -3559,7 +3559,7 @@
     </row>
     <row r="78">
       <c r="A78" s="200">
-        <f>Inquilini!A2</f>
+        <f>Inquilini!B2</f>
         <v/>
       </c>
       <c r="B78" s="199" t="n">
@@ -3591,7 +3591,7 @@
     </row>
     <row r="80">
       <c r="A80" s="200">
-        <f>Inquilini!A3</f>
+        <f>Inquilini!B3</f>
         <v/>
       </c>
       <c r="B80" s="199" t="n">
@@ -3621,7 +3621,7 @@
     </row>
     <row r="82">
       <c r="A82" s="200">
-        <f>Inquilini!A4</f>
+        <f>Inquilini!B4</f>
         <v/>
       </c>
       <c r="B82" s="199" t="n">
@@ -3651,7 +3651,7 @@
     </row>
     <row r="84">
       <c r="A84" s="200">
-        <f>Inquilini!A5</f>
+        <f>Inquilini!B5</f>
         <v/>
       </c>
       <c r="B84" s="199" t="n">
@@ -3681,7 +3681,7 @@
     </row>
     <row r="86">
       <c r="A86" s="200">
-        <f>Inquilini!A6</f>
+        <f>Inquilini!B6</f>
         <v/>
       </c>
       <c r="B86" s="199" t="n">
@@ -3711,7 +3711,7 @@
     </row>
     <row r="88">
       <c r="A88" s="200">
-        <f>Inquilini!A7</f>
+        <f>Inquilini!B7</f>
         <v/>
       </c>
       <c r="B88" s="199" t="n">
@@ -3741,7 +3741,7 @@
     </row>
     <row r="90">
       <c r="A90" s="200">
-        <f>Inquilini!A8</f>
+        <f>Inquilini!B8</f>
         <v/>
       </c>
       <c r="B90" s="199" t="n">
@@ -3771,7 +3771,7 @@
     </row>
     <row r="92">
       <c r="A92" s="200">
-        <f>Inquilini!A9</f>
+        <f>Inquilini!B9</f>
         <v/>
       </c>
       <c r="B92" s="199" t="n">
@@ -3801,7 +3801,7 @@
     </row>
     <row r="94">
       <c r="A94" s="200">
-        <f>Inquilini!A10</f>
+        <f>Inquilini!B10</f>
         <v/>
       </c>
       <c r="B94" s="199" t="n">
@@ -3942,7 +3942,7 @@
     </row>
     <row r="103">
       <c r="A103" s="200">
-        <f>Inquilini!A2</f>
+        <f>Inquilini!B2</f>
         <v/>
       </c>
       <c r="B103" s="85">
@@ -3971,7 +3971,7 @@
     </row>
     <row r="105">
       <c r="A105" s="200">
-        <f>Inquilini!A3</f>
+        <f>Inquilini!B3</f>
         <v/>
       </c>
       <c r="B105" s="85">
@@ -4000,7 +4000,7 @@
     </row>
     <row r="107">
       <c r="A107" s="200">
-        <f>Inquilini!A4</f>
+        <f>Inquilini!B4</f>
         <v/>
       </c>
       <c r="B107" s="85">
@@ -4029,7 +4029,7 @@
     </row>
     <row r="109">
       <c r="A109" s="200">
-        <f>Inquilini!A5</f>
+        <f>Inquilini!B5</f>
         <v/>
       </c>
       <c r="B109" s="85">
@@ -4059,7 +4059,7 @@
     </row>
     <row r="111">
       <c r="A111" s="200">
-        <f>Inquilini!A6</f>
+        <f>Inquilini!B6</f>
         <v/>
       </c>
       <c r="B111" s="85">
@@ -4088,7 +4088,7 @@
     </row>
     <row r="113">
       <c r="A113" s="200">
-        <f>Inquilini!A7</f>
+        <f>Inquilini!B7</f>
         <v/>
       </c>
       <c r="B113" s="85">
@@ -4117,7 +4117,7 @@
     </row>
     <row r="115">
       <c r="A115" s="200">
-        <f>Inquilini!A8</f>
+        <f>Inquilini!B8</f>
         <v/>
       </c>
       <c r="B115" s="85">
@@ -4147,7 +4147,7 @@
     </row>
     <row r="117">
       <c r="A117" s="200">
-        <f>Inquilini!A9</f>
+        <f>Inquilini!B9</f>
         <v/>
       </c>
       <c r="B117" s="85">
@@ -4176,7 +4176,7 @@
     </row>
     <row r="119">
       <c r="A119" s="200">
-        <f>Inquilini!A10</f>
+        <f>Inquilini!B10</f>
         <v/>
       </c>
       <c r="B119" s="85">
@@ -4347,7 +4347,7 @@
     </row>
     <row r="130">
       <c r="A130" s="200">
-        <f>Inquilini!A2</f>
+        <f>Inquilini!B2</f>
         <v/>
       </c>
       <c r="B130" s="330" t="n">
@@ -4384,7 +4384,7 @@
     </row>
     <row r="132" ht="14.4" customHeight="1">
       <c r="A132" s="200">
-        <f>Inquilini!A3</f>
+        <f>Inquilini!B3</f>
         <v/>
       </c>
       <c r="B132" s="330" t="n">
@@ -4419,7 +4419,7 @@
     </row>
     <row r="134">
       <c r="A134" s="200">
-        <f>Inquilini!A4</f>
+        <f>Inquilini!B4</f>
         <v/>
       </c>
       <c r="B134" s="330" t="n">
@@ -4454,7 +4454,7 @@
     </row>
     <row r="136" ht="14.4" customHeight="1">
       <c r="A136" s="200">
-        <f>Inquilini!A5</f>
+        <f>Inquilini!B5</f>
         <v/>
       </c>
       <c r="B136" s="330" t="n">
@@ -4490,7 +4490,7 @@
     </row>
     <row r="138" ht="14.4" customHeight="1">
       <c r="A138" s="200">
-        <f>Inquilini!A6</f>
+        <f>Inquilini!B6</f>
         <v/>
       </c>
       <c r="B138" s="330" t="n">
@@ -4525,7 +4525,7 @@
     </row>
     <row r="140">
       <c r="A140" s="200">
-        <f>Inquilini!A7</f>
+        <f>Inquilini!B7</f>
         <v/>
       </c>
       <c r="B140" s="330" t="n">
@@ -4561,7 +4561,7 @@
     </row>
     <row r="142" ht="14.4" customHeight="1">
       <c r="A142" s="200">
-        <f>Inquilini!A8</f>
+        <f>Inquilini!B8</f>
         <v/>
       </c>
       <c r="B142" s="330" t="n">
@@ -4596,7 +4596,7 @@
     </row>
     <row r="144">
       <c r="A144" s="200">
-        <f>Inquilini!A9</f>
+        <f>Inquilini!B9</f>
         <v/>
       </c>
       <c r="B144" s="330" t="n">
@@ -4631,7 +4631,7 @@
     </row>
     <row r="146">
       <c r="A146" s="200">
-        <f>Inquilini!A10</f>
+        <f>Inquilini!B10</f>
         <v/>
       </c>
       <c r="B146" s="330" t="n">
@@ -4824,7 +4824,7 @@
     </row>
     <row r="158">
       <c r="A158" s="200">
-        <f>Inquilini!A2</f>
+        <f>Inquilini!B2</f>
         <v/>
       </c>
       <c r="B158" s="85">
@@ -4851,7 +4851,7 @@
     </row>
     <row r="160">
       <c r="A160" s="200">
-        <f>Inquilini!A3</f>
+        <f>Inquilini!B3</f>
         <v/>
       </c>
       <c r="B160" s="85">
@@ -4878,7 +4878,7 @@
     </row>
     <row r="162">
       <c r="A162" s="200">
-        <f>Inquilini!A4</f>
+        <f>Inquilini!B4</f>
         <v/>
       </c>
       <c r="B162" s="85">
@@ -4906,7 +4906,7 @@
     </row>
     <row r="164">
       <c r="A164" s="200">
-        <f>Inquilini!A5</f>
+        <f>Inquilini!B5</f>
         <v/>
       </c>
       <c r="B164" s="85">
@@ -4934,7 +4934,7 @@
     </row>
     <row r="166">
       <c r="A166" s="200">
-        <f>Inquilini!A6</f>
+        <f>Inquilini!B6</f>
         <v/>
       </c>
       <c r="B166" s="85">
@@ -4961,7 +4961,7 @@
     </row>
     <row r="168">
       <c r="A168" s="200">
-        <f>Inquilini!A7</f>
+        <f>Inquilini!B7</f>
         <v/>
       </c>
       <c r="B168" s="85">
@@ -4988,7 +4988,7 @@
     </row>
     <row r="170">
       <c r="A170" s="200">
-        <f>Inquilini!A8</f>
+        <f>Inquilini!B8</f>
         <v/>
       </c>
       <c r="B170" s="85">
@@ -5016,7 +5016,7 @@
     </row>
     <row r="172">
       <c r="A172" s="200">
-        <f>Inquilini!A9</f>
+        <f>Inquilini!B9</f>
         <v/>
       </c>
       <c r="B172" s="85">
@@ -5043,7 +5043,7 @@
     </row>
     <row r="174" ht="13.8" customHeight="1" thickBot="1">
       <c r="A174" s="200">
-        <f>Inquilini!A10</f>
+        <f>Inquilini!B10</f>
         <v/>
       </c>
       <c r="B174" s="85">
@@ -5191,7 +5191,7 @@
     </row>
     <row r="182">
       <c r="A182" s="200">
-        <f>Inquilini!A2</f>
+        <f>Inquilini!B2</f>
         <v/>
       </c>
       <c r="B182" s="330" t="n">
@@ -5226,7 +5226,7 @@
     </row>
     <row r="184">
       <c r="A184" s="200">
-        <f>Inquilini!A3</f>
+        <f>Inquilini!B3</f>
         <v/>
       </c>
       <c r="B184" s="330" t="n">
@@ -5261,7 +5261,7 @@
     </row>
     <row r="186">
       <c r="A186" s="200">
-        <f>Inquilini!A4</f>
+        <f>Inquilini!B4</f>
         <v/>
       </c>
       <c r="B186" s="341" t="n">
@@ -5302,7 +5302,7 @@
     </row>
     <row r="188">
       <c r="A188" s="200">
-        <f>Inquilini!A5</f>
+        <f>Inquilini!B5</f>
         <v/>
       </c>
       <c r="B188" s="330" t="n">
@@ -5337,7 +5337,7 @@
     </row>
     <row r="190">
       <c r="A190" s="200">
-        <f>Inquilini!A6</f>
+        <f>Inquilini!B6</f>
         <v/>
       </c>
       <c r="B190" s="330" t="n">
@@ -5372,7 +5372,7 @@
     </row>
     <row r="192">
       <c r="A192" s="200">
-        <f>Inquilini!A7</f>
+        <f>Inquilini!B7</f>
         <v/>
       </c>
       <c r="B192" s="330" t="n">
@@ -5407,7 +5407,7 @@
     </row>
     <row r="194">
       <c r="A194" s="200">
-        <f>Inquilini!A8</f>
+        <f>Inquilini!B8</f>
         <v/>
       </c>
       <c r="B194" s="330" t="n">
@@ -5445,7 +5445,7 @@
     </row>
     <row r="196">
       <c r="A196" s="200">
-        <f>Inquilini!A9</f>
+        <f>Inquilini!B9</f>
         <v/>
       </c>
       <c r="B196" s="330" t="n">
@@ -5483,7 +5483,7 @@
     </row>
     <row r="198">
       <c r="A198" s="200">
-        <f>Inquilini!A10</f>
+        <f>Inquilini!B10</f>
         <v/>
       </c>
       <c r="B198" s="330" t="n">
@@ -5611,7 +5611,7 @@
     </row>
     <row r="205">
       <c r="A205" s="200">
-        <f>Inquilini!A2</f>
+        <f>Inquilini!B2</f>
         <v/>
       </c>
       <c r="B205" s="279">
@@ -5640,7 +5640,7 @@
     </row>
     <row r="207">
       <c r="A207" s="200">
-        <f>Inquilini!A3</f>
+        <f>Inquilini!B3</f>
         <v/>
       </c>
       <c r="B207" s="279">
@@ -5669,7 +5669,7 @@
     </row>
     <row r="209">
       <c r="A209" s="72">
-        <f>Inquilini!A4</f>
+        <f>Inquilini!B4</f>
         <v/>
       </c>
       <c r="B209" s="279">
@@ -5698,7 +5698,7 @@
     </row>
     <row r="211">
       <c r="A211" s="200">
-        <f>Inquilini!A5</f>
+        <f>Inquilini!B5</f>
         <v/>
       </c>
       <c r="B211" s="279">
@@ -5727,7 +5727,7 @@
     </row>
     <row r="213">
       <c r="A213" s="200">
-        <f>Inquilini!A6</f>
+        <f>Inquilini!B6</f>
         <v/>
       </c>
       <c r="B213" s="279">
@@ -5756,7 +5756,7 @@
     </row>
     <row r="215">
       <c r="A215" s="200">
-        <f>Inquilini!A7</f>
+        <f>Inquilini!B7</f>
         <v/>
       </c>
       <c r="B215" s="279">
@@ -5785,7 +5785,7 @@
     </row>
     <row r="217">
       <c r="A217" s="200">
-        <f>Inquilini!A8</f>
+        <f>Inquilini!B8</f>
         <v/>
       </c>
       <c r="B217" s="279">
@@ -5814,7 +5814,7 @@
     </row>
     <row r="219">
       <c r="A219" s="200">
-        <f>Inquilini!A9</f>
+        <f>Inquilini!B9</f>
         <v/>
       </c>
       <c r="B219" s="279">
@@ -5843,7 +5843,7 @@
     </row>
     <row r="221">
       <c r="A221" s="200">
-        <f>Inquilini!A10</f>
+        <f>Inquilini!B10</f>
         <v/>
       </c>
       <c r="B221" s="279">
@@ -6050,7 +6050,7 @@
     </row>
     <row r="229">
       <c r="A229" s="200">
-        <f>Inquilini!A2</f>
+        <f>Inquilini!B2</f>
         <v/>
       </c>
       <c r="B229" s="126">
@@ -6105,7 +6105,7 @@
     </row>
     <row r="231">
       <c r="A231" s="200">
-        <f>Inquilini!A3</f>
+        <f>Inquilini!B3</f>
         <v/>
       </c>
       <c r="B231" s="126">
@@ -6160,7 +6160,7 @@
     </row>
     <row r="233">
       <c r="A233" s="200">
-        <f>Inquilini!A4</f>
+        <f>Inquilini!B4</f>
         <v/>
       </c>
       <c r="B233" s="126">
@@ -6215,7 +6215,7 @@
     </row>
     <row r="235">
       <c r="A235" s="200">
-        <f>Inquilini!A5</f>
+        <f>Inquilini!B5</f>
         <v/>
       </c>
       <c r="B235" s="126">
@@ -6270,7 +6270,7 @@
     </row>
     <row r="237">
       <c r="A237" s="200">
-        <f>Inquilini!A6</f>
+        <f>Inquilini!B6</f>
         <v/>
       </c>
       <c r="B237" s="126">
@@ -6325,7 +6325,7 @@
     </row>
     <row r="239">
       <c r="A239" s="200">
-        <f>Inquilini!A7</f>
+        <f>Inquilini!B7</f>
         <v/>
       </c>
       <c r="B239" s="126">
@@ -6380,7 +6380,7 @@
     </row>
     <row r="241">
       <c r="A241" s="200">
-        <f>Inquilini!A8</f>
+        <f>Inquilini!B8</f>
         <v/>
       </c>
       <c r="B241" s="126">
@@ -6436,7 +6436,7 @@
     </row>
     <row r="243">
       <c r="A243" s="200">
-        <f>Inquilini!A9</f>
+        <f>Inquilini!B9</f>
         <v/>
       </c>
       <c r="B243" s="126">
@@ -6493,7 +6493,7 @@
     </row>
     <row r="245">
       <c r="A245" s="200">
-        <f>Inquilini!A10</f>
+        <f>Inquilini!B10</f>
         <v/>
       </c>
       <c r="B245" s="126">
@@ -6852,7 +6852,7 @@
     </row>
     <row r="259">
       <c r="A259" s="200">
-        <f>Inquilini!A2</f>
+        <f>Inquilini!B2</f>
         <v/>
       </c>
       <c r="B259" s="126" t="n"/>
@@ -6890,7 +6890,7 @@
     </row>
     <row r="261" ht="14.4" customHeight="1">
       <c r="A261" s="200">
-        <f>Inquilini!A3</f>
+        <f>Inquilini!B3</f>
         <v/>
       </c>
       <c r="B261" s="126" t="n"/>
@@ -6945,7 +6945,7 @@
     </row>
     <row r="263">
       <c r="A263" s="200">
-        <f>Inquilini!A4</f>
+        <f>Inquilini!B4</f>
         <v/>
       </c>
       <c r="B263" s="126" t="n"/>
@@ -6985,7 +6985,7 @@
     </row>
     <row r="265" ht="14.4" customHeight="1">
       <c r="A265" s="200">
-        <f>Inquilini!A5</f>
+        <f>Inquilini!B5</f>
         <v/>
       </c>
       <c r="B265" s="126" t="n"/>
@@ -7045,7 +7045,7 @@
     </row>
     <row r="267" ht="14.4" customHeight="1">
       <c r="A267" s="200">
-        <f>Inquilini!A6</f>
+        <f>Inquilini!B6</f>
         <v/>
       </c>
       <c r="B267" s="126" t="n"/>
@@ -7105,7 +7105,7 @@
     </row>
     <row r="269">
       <c r="A269" s="200">
-        <f>Inquilini!A7</f>
+        <f>Inquilini!B7</f>
         <v/>
       </c>
       <c r="B269" s="126" t="n"/>
@@ -7145,7 +7145,7 @@
     </row>
     <row r="271" ht="14.4" customHeight="1">
       <c r="A271" s="200">
-        <f>Inquilini!A8</f>
+        <f>Inquilini!B8</f>
         <v/>
       </c>
       <c r="B271" s="126" t="n"/>
@@ -7199,7 +7199,7 @@
     </row>
     <row r="273" ht="14.4" customHeight="1">
       <c r="A273" s="200">
-        <f>Inquilini!A9</f>
+        <f>Inquilini!B9</f>
         <v/>
       </c>
       <c r="B273" s="126" t="n"/>
@@ -7248,7 +7248,7 @@
     </row>
     <row r="275">
       <c r="A275" s="200">
-        <f>Inquilini!A10</f>
+        <f>Inquilini!B10</f>
         <v/>
       </c>
       <c r="B275" s="126" t="n"/>

</xml_diff>